<commit_message>
To Demo again. 2nd page Done
</commit_message>
<xml_diff>
--- a/backend/python/templates/UNIRRIG_Template.xlsx
+++ b/backend/python/templates/UNIRRIG_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Videos\FAAS SYSTEM\backend\python\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86F1CEFF-B62F-4D34-B1AB-661D6B353A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6FEBDF5-D34A-4176-A5E3-4D3D4A9950F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$K$66</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">Sheet2!$A$1:$M$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Sheet2!$A$1:$M$72</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="127">
   <si>
     <t>PROPERTY INDEX NO.</t>
   </si>
@@ -430,6 +430,15 @@
   </si>
   <si>
     <t>REENA N. AURIN, REA 0005811</t>
+  </si>
+  <si>
+    <t>FOR 20</t>
+  </si>
+  <si>
+    <t>BY</t>
+  </si>
+  <si>
+    <t>PREVIOUS OWNER</t>
   </si>
 </sst>
 </file>
@@ -799,7 +808,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="280">
+  <cellXfs count="282">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1117,9 +1126,6 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1137,55 +1143,338 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="7"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="4" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1193,14 +1482,12 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1208,314 +1495,31 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="4" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="15" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="14" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="4" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" indent="7"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="15" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="14" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="15" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="14" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
@@ -1907,32 +1911,32 @@
     <row r="1" spans="1:11" ht="3.75" customHeight="1"/>
     <row r="2" spans="1:11" hidden="1"/>
     <row r="3" spans="1:11">
-      <c r="H3" s="171" t="s">
+      <c r="H3" s="246" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="145"/>
-      <c r="J3" s="150"/>
-      <c r="K3" s="259"/>
+      <c r="I3" s="179"/>
+      <c r="J3" s="212"/>
+      <c r="K3" s="224"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="172" t="s">
+      <c r="A4" s="247" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="145"/>
-      <c r="C4" s="145"/>
-      <c r="D4" s="145"/>
-      <c r="E4" s="145"/>
+      <c r="B4" s="179"/>
+      <c r="C4" s="179"/>
+      <c r="D4" s="179"/>
+      <c r="E4" s="179"/>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="175" t="s">
+      <c r="A5" s="218" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="145"/>
-      <c r="C5" s="150"/>
-      <c r="D5" s="259"/>
-      <c r="E5" s="259"/>
-      <c r="F5" s="259"/>
-      <c r="G5" s="259"/>
+      <c r="B5" s="179"/>
+      <c r="C5" s="212"/>
+      <c r="D5" s="224"/>
+      <c r="E5" s="224"/>
+      <c r="F5" s="224"/>
+      <c r="G5" s="224"/>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="10"/>
@@ -1943,154 +1947,154 @@
     </row>
     <row r="7" spans="1:11" ht="18.75">
       <c r="A7" s="95"/>
-      <c r="C7" s="260" t="s">
+      <c r="C7" s="251" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="145"/>
-      <c r="E7" s="145"/>
-      <c r="F7" s="145"/>
-      <c r="G7" s="145"/>
-      <c r="H7" s="145"/>
-      <c r="I7" s="145"/>
+      <c r="D7" s="179"/>
+      <c r="E7" s="179"/>
+      <c r="F7" s="179"/>
+      <c r="G7" s="179"/>
+      <c r="H7" s="179"/>
+      <c r="I7" s="179"/>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="261" t="s">
+      <c r="A8" s="225" t="s">
         <v>118</v>
       </c>
-      <c r="B8" s="145"/>
-      <c r="C8" s="145"/>
-      <c r="D8" s="145"/>
-      <c r="E8" s="145"/>
-      <c r="F8" s="145"/>
-      <c r="G8" s="145"/>
-      <c r="H8" s="145"/>
-      <c r="I8" s="145"/>
-      <c r="J8" s="145"/>
-      <c r="K8" s="145"/>
+      <c r="B8" s="179"/>
+      <c r="C8" s="179"/>
+      <c r="D8" s="179"/>
+      <c r="E8" s="179"/>
+      <c r="F8" s="179"/>
+      <c r="G8" s="179"/>
+      <c r="H8" s="179"/>
+      <c r="I8" s="179"/>
+      <c r="J8" s="179"/>
+      <c r="K8" s="179"/>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="150"/>
-      <c r="C11" s="259"/>
-      <c r="D11" s="259"/>
-      <c r="E11" s="259"/>
-      <c r="F11" s="259"/>
-      <c r="G11" s="259"/>
-      <c r="H11" s="150"/>
-      <c r="I11" s="259"/>
-      <c r="J11" s="259"/>
-      <c r="K11" s="259"/>
+      <c r="B11" s="212"/>
+      <c r="C11" s="224"/>
+      <c r="D11" s="224"/>
+      <c r="E11" s="224"/>
+      <c r="F11" s="224"/>
+      <c r="G11" s="224"/>
+      <c r="H11" s="212"/>
+      <c r="I11" s="224"/>
+      <c r="J11" s="224"/>
+      <c r="K11" s="224"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="189" t="s">
+      <c r="A12" s="226" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="145"/>
-      <c r="C12" s="145"/>
-      <c r="D12" s="145"/>
-      <c r="E12" s="145"/>
-      <c r="F12" s="145"/>
-      <c r="G12" s="145"/>
-      <c r="H12" s="145"/>
-      <c r="I12" s="145"/>
-      <c r="J12" s="145"/>
-      <c r="K12" s="145"/>
+      <c r="B12" s="179"/>
+      <c r="C12" s="179"/>
+      <c r="D12" s="179"/>
+      <c r="E12" s="179"/>
+      <c r="F12" s="179"/>
+      <c r="G12" s="179"/>
+      <c r="H12" s="179"/>
+      <c r="I12" s="179"/>
+      <c r="J12" s="179"/>
+      <c r="K12" s="179"/>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B13" s="150"/>
-      <c r="C13" s="259"/>
-      <c r="D13" s="259"/>
-      <c r="E13" s="259"/>
-      <c r="F13" s="259"/>
-      <c r="G13" s="259"/>
-      <c r="H13" s="150"/>
-      <c r="I13" s="259"/>
-      <c r="J13" s="259"/>
-      <c r="K13" s="259"/>
+      <c r="B13" s="212"/>
+      <c r="C13" s="224"/>
+      <c r="D13" s="224"/>
+      <c r="E13" s="224"/>
+      <c r="F13" s="224"/>
+      <c r="G13" s="224"/>
+      <c r="H13" s="212"/>
+      <c r="I13" s="224"/>
+      <c r="J13" s="224"/>
+      <c r="K13" s="224"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="168" t="s">
+      <c r="A14" s="255" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="145"/>
-      <c r="C14" s="145"/>
-      <c r="D14" s="145"/>
-      <c r="E14" s="145"/>
-      <c r="F14" s="145"/>
-      <c r="G14" s="145"/>
-      <c r="H14" s="145"/>
-      <c r="I14" s="145"/>
-      <c r="J14" s="145"/>
-      <c r="K14" s="145"/>
+      <c r="B14" s="179"/>
+      <c r="C14" s="179"/>
+      <c r="D14" s="179"/>
+      <c r="E14" s="179"/>
+      <c r="F14" s="179"/>
+      <c r="G14" s="179"/>
+      <c r="H14" s="179"/>
+      <c r="I14" s="179"/>
+      <c r="J14" s="179"/>
+      <c r="K14" s="179"/>
     </row>
     <row r="16" spans="1:11" ht="18">
-      <c r="A16" s="159" t="s">
+      <c r="A16" s="257" t="s">
         <v>8</v>
       </c>
-      <c r="B16" s="145"/>
-      <c r="C16" s="145"/>
-      <c r="D16" s="145"/>
-      <c r="E16" s="145"/>
-      <c r="F16" s="145"/>
-      <c r="G16" s="145"/>
-      <c r="H16" s="145"/>
-      <c r="I16" s="145"/>
-      <c r="J16" s="145"/>
-      <c r="K16" s="145"/>
+      <c r="B16" s="179"/>
+      <c r="C16" s="179"/>
+      <c r="D16" s="179"/>
+      <c r="E16" s="179"/>
+      <c r="F16" s="179"/>
+      <c r="G16" s="179"/>
+      <c r="H16" s="179"/>
+      <c r="I16" s="179"/>
+      <c r="J16" s="179"/>
+      <c r="K16" s="179"/>
     </row>
     <row r="17" spans="1:11" ht="18">
-      <c r="A17" s="166" t="s">
+      <c r="A17" s="194" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="145"/>
-      <c r="C17" s="147"/>
-      <c r="D17" s="262"/>
-      <c r="E17" s="262"/>
+      <c r="B17" s="179"/>
+      <c r="C17" s="166"/>
+      <c r="D17" s="261"/>
+      <c r="E17" s="261"/>
       <c r="F17" s="20"/>
-      <c r="G17" s="147"/>
-      <c r="H17" s="259"/>
-      <c r="I17" s="147"/>
-      <c r="J17" s="259"/>
-      <c r="K17" s="259"/>
+      <c r="G17" s="166"/>
+      <c r="H17" s="224"/>
+      <c r="I17" s="166"/>
+      <c r="J17" s="224"/>
+      <c r="K17" s="224"/>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="21"/>
       <c r="B18" s="21"/>
-      <c r="C18" s="176" t="s">
+      <c r="C18" s="185" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="145"/>
-      <c r="E18" s="145"/>
+      <c r="D18" s="179"/>
+      <c r="E18" s="179"/>
       <c r="F18" s="21"/>
-      <c r="G18" s="176" t="s">
+      <c r="G18" s="185" t="s">
         <v>11</v>
       </c>
-      <c r="H18" s="145"/>
-      <c r="I18" s="176" t="s">
+      <c r="H18" s="179"/>
+      <c r="I18" s="185" t="s">
         <v>12</v>
       </c>
-      <c r="J18" s="145"/>
-      <c r="K18" s="145"/>
+      <c r="J18" s="179"/>
+      <c r="K18" s="179"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="166" t="s">
+      <c r="A19" s="194" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="145"/>
-      <c r="C19" s="150"/>
-      <c r="D19" s="259"/>
-      <c r="E19" s="259"/>
+      <c r="B19" s="179"/>
+      <c r="C19" s="212"/>
+      <c r="D19" s="224"/>
+      <c r="E19" s="224"/>
       <c r="F19" s="19"/>
       <c r="G19" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="H19" s="147"/>
-      <c r="I19" s="147"/>
+      <c r="H19" s="166"/>
+      <c r="I19" s="166"/>
       <c r="J19" s="21" t="s">
         <v>14</v>
       </c>
@@ -2117,95 +2121,95 @@
       <c r="A21" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="B21" s="150"/>
-      <c r="C21" s="259"/>
-      <c r="D21" s="259"/>
-      <c r="E21" s="259"/>
-      <c r="F21" s="259"/>
-      <c r="G21" s="259"/>
+      <c r="B21" s="212"/>
+      <c r="C21" s="224"/>
+      <c r="D21" s="224"/>
+      <c r="E21" s="224"/>
+      <c r="F21" s="224"/>
+      <c r="G21" s="224"/>
       <c r="H21" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="I21" s="150"/>
-      <c r="J21" s="259"/>
-      <c r="K21" s="259"/>
+      <c r="I21" s="212"/>
+      <c r="J21" s="224"/>
+      <c r="K21" s="224"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="179"/>
-      <c r="C22" s="263"/>
-      <c r="D22" s="263"/>
-      <c r="E22" s="263"/>
-      <c r="F22" s="263"/>
-      <c r="G22" s="263"/>
+      <c r="B22" s="229"/>
+      <c r="C22" s="230"/>
+      <c r="D22" s="230"/>
+      <c r="E22" s="230"/>
+      <c r="F22" s="230"/>
+      <c r="G22" s="230"/>
       <c r="H22" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="I22" s="179"/>
-      <c r="J22" s="263"/>
-      <c r="K22" s="263"/>
+      <c r="I22" s="229"/>
+      <c r="J22" s="230"/>
+      <c r="K22" s="230"/>
     </row>
     <row r="23" spans="1:11">
-      <c r="A23" s="170" t="s">
+      <c r="A23" s="256" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="145"/>
-      <c r="C23" s="145"/>
-      <c r="D23" s="145"/>
-      <c r="E23" s="145"/>
-      <c r="F23" s="145"/>
-      <c r="G23" s="145"/>
-      <c r="H23" s="145"/>
-      <c r="I23" s="145"/>
-      <c r="J23" s="145"/>
-      <c r="K23" s="145"/>
+      <c r="B23" s="179"/>
+      <c r="C23" s="179"/>
+      <c r="D23" s="179"/>
+      <c r="E23" s="179"/>
+      <c r="F23" s="179"/>
+      <c r="G23" s="179"/>
+      <c r="H23" s="179"/>
+      <c r="I23" s="179"/>
+      <c r="J23" s="179"/>
+      <c r="K23" s="179"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="185"/>
-      <c r="B24" s="141"/>
-      <c r="C24" s="141"/>
-      <c r="D24" s="141"/>
-      <c r="E24" s="141"/>
-      <c r="F24" s="141"/>
-      <c r="G24" s="141"/>
-      <c r="H24" s="141"/>
-      <c r="I24" s="141"/>
-      <c r="J24" s="141"/>
-      <c r="K24" s="141"/>
+      <c r="A24" s="244"/>
+      <c r="B24" s="159"/>
+      <c r="C24" s="159"/>
+      <c r="D24" s="159"/>
+      <c r="E24" s="159"/>
+      <c r="F24" s="159"/>
+      <c r="G24" s="159"/>
+      <c r="H24" s="159"/>
+      <c r="I24" s="159"/>
+      <c r="J24" s="159"/>
+      <c r="K24" s="159"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="177" t="s">
+      <c r="A25" s="168" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="178"/>
-      <c r="C25" s="178"/>
-      <c r="D25" s="178"/>
-      <c r="E25" s="178"/>
-      <c r="F25" s="178"/>
-      <c r="G25" s="178"/>
-      <c r="H25" s="178"/>
-      <c r="I25" s="178"/>
-      <c r="J25" s="178"/>
-      <c r="K25" s="178"/>
+      <c r="B25" s="138"/>
+      <c r="C25" s="138"/>
+      <c r="D25" s="138"/>
+      <c r="E25" s="138"/>
+      <c r="F25" s="138"/>
+      <c r="G25" s="138"/>
+      <c r="H25" s="138"/>
+      <c r="I25" s="138"/>
+      <c r="J25" s="138"/>
+      <c r="K25" s="138"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="188" t="s">
+      <c r="A26" s="245" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="138"/>
-      <c r="C26" s="139"/>
+      <c r="B26" s="140"/>
+      <c r="C26" s="141"/>
       <c r="D26" s="26"/>
-      <c r="E26" s="191" t="s">
+      <c r="E26" s="223" t="s">
         <v>24</v>
       </c>
-      <c r="F26" s="138"/>
-      <c r="G26" s="138"/>
-      <c r="H26" s="138"/>
-      <c r="I26" s="138"/>
-      <c r="J26" s="138"/>
-      <c r="K26" s="138"/>
+      <c r="F26" s="140"/>
+      <c r="G26" s="140"/>
+      <c r="H26" s="140"/>
+      <c r="I26" s="140"/>
+      <c r="J26" s="140"/>
+      <c r="K26" s="140"/>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="27" t="s">
@@ -2218,10 +2222,10 @@
         <v>27</v>
       </c>
       <c r="D27" s="48"/>
-      <c r="E27" s="183" t="s">
+      <c r="E27" s="238" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="139"/>
+      <c r="F27" s="141"/>
       <c r="G27" s="49" t="s">
         <v>26</v>
       </c>
@@ -2231,18 +2235,18 @@
       <c r="I27" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="J27" s="194" t="s">
+      <c r="J27" s="237" t="s">
         <v>30</v>
       </c>
-      <c r="K27" s="139"/>
+      <c r="K27" s="141"/>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="28"/>
       <c r="B28" s="28"/>
       <c r="C28" s="28"/>
       <c r="D28" s="26"/>
-      <c r="E28" s="146"/>
-      <c r="F28" s="264"/>
+      <c r="E28" s="260"/>
+      <c r="F28" s="249"/>
       <c r="G28" s="76"/>
       <c r="H28" s="77"/>
       <c r="I28" s="78" t="str">
@@ -2262,16 +2266,16 @@
 )</f>
         <v/>
       </c>
-      <c r="J28" s="143"/>
-      <c r="K28" s="265"/>
+      <c r="J28" s="239"/>
+      <c r="K28" s="240"/>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="31"/>
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
       <c r="D29" s="26"/>
-      <c r="E29" s="161"/>
-      <c r="F29" s="266"/>
+      <c r="E29" s="253"/>
+      <c r="F29" s="254"/>
       <c r="G29" s="76"/>
       <c r="H29" s="79"/>
       <c r="I29" s="78" t="str">
@@ -2291,16 +2295,16 @@
 )</f>
         <v/>
       </c>
-      <c r="J29" s="143"/>
-      <c r="K29" s="265"/>
+      <c r="J29" s="239"/>
+      <c r="K29" s="240"/>
     </row>
     <row r="30" spans="1:11" hidden="1">
       <c r="A30" s="28"/>
       <c r="B30" s="28"/>
       <c r="C30" s="28"/>
       <c r="D30" s="26"/>
-      <c r="E30" s="149"/>
-      <c r="F30" s="267"/>
+      <c r="E30" s="263"/>
+      <c r="F30" s="228"/>
       <c r="G30" s="76"/>
       <c r="H30" s="80"/>
       <c r="I30" s="78" t="str">
@@ -2320,29 +2324,29 @@
 )</f>
         <v/>
       </c>
-      <c r="J30" s="143"/>
-      <c r="K30" s="265"/>
+      <c r="J30" s="239"/>
+      <c r="K30" s="240"/>
     </row>
     <row r="31" spans="1:11" hidden="1">
       <c r="A31" s="28"/>
       <c r="B31" s="28"/>
       <c r="C31" s="28"/>
       <c r="D31" s="26"/>
-      <c r="E31" s="167"/>
-      <c r="F31" s="264"/>
+      <c r="E31" s="248"/>
+      <c r="F31" s="249"/>
       <c r="G31" s="76"/>
       <c r="H31" s="81"/>
       <c r="I31" s="78"/>
-      <c r="J31" s="143"/>
-      <c r="K31" s="265"/>
+      <c r="J31" s="239"/>
+      <c r="K31" s="240"/>
     </row>
     <row r="32" spans="1:11" hidden="1">
       <c r="A32" s="28"/>
       <c r="B32" s="28"/>
       <c r="C32" s="28"/>
       <c r="D32" s="26"/>
-      <c r="E32" s="167"/>
-      <c r="F32" s="264"/>
+      <c r="E32" s="248"/>
+      <c r="F32" s="249"/>
       <c r="G32" s="76"/>
       <c r="H32" s="81" t="s">
         <v>39</v>
@@ -2364,16 +2368,16 @@
 )</f>
         <v/>
       </c>
-      <c r="J32" s="152"/>
-      <c r="K32" s="264"/>
+      <c r="J32" s="265"/>
+      <c r="K32" s="249"/>
     </row>
     <row r="33" spans="1:11" ht="14.25" customHeight="1">
       <c r="A33" s="28"/>
       <c r="B33" s="28"/>
       <c r="C33" s="28"/>
       <c r="D33" s="26"/>
-      <c r="E33" s="167"/>
-      <c r="F33" s="264"/>
+      <c r="E33" s="248"/>
+      <c r="F33" s="249"/>
       <c r="G33" s="76"/>
       <c r="H33" s="81" t="s">
         <v>39</v>
@@ -2395,16 +2399,16 @@
 )</f>
         <v/>
       </c>
-      <c r="J33" s="152"/>
-      <c r="K33" s="264"/>
+      <c r="J33" s="265"/>
+      <c r="K33" s="249"/>
     </row>
     <row r="34" spans="1:11" hidden="1">
       <c r="A34" s="28"/>
       <c r="B34" s="28"/>
       <c r="C34" s="28"/>
       <c r="D34" s="26"/>
-      <c r="E34" s="182"/>
-      <c r="F34" s="139"/>
+      <c r="E34" s="205"/>
+      <c r="F34" s="141"/>
       <c r="G34" s="67"/>
       <c r="H34" s="30" t="s">
         <v>39</v>
@@ -2426,26 +2430,26 @@
 )</f>
         <v/>
       </c>
-      <c r="J34" s="193" t="str">
+      <c r="J34" s="233" t="str">
         <f t="shared" ref="J34" si="0">IFERROR(MROUND(G34*I34,10),"")</f>
         <v/>
       </c>
-      <c r="K34" s="139"/>
+      <c r="K34" s="141"/>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="28"/>
       <c r="B35" s="28"/>
       <c r="C35" s="28"/>
       <c r="D35" s="26"/>
-      <c r="E35" s="154" t="s">
+      <c r="E35" s="250" t="s">
         <v>31</v>
       </c>
-      <c r="F35" s="139"/>
+      <c r="F35" s="141"/>
       <c r="G35" s="29"/>
       <c r="H35" s="30"/>
       <c r="I35" s="30"/>
-      <c r="J35" s="184"/>
-      <c r="K35" s="268"/>
+      <c r="J35" s="242"/>
+      <c r="K35" s="243"/>
     </row>
     <row r="36" spans="1:11">
       <c r="A36" s="32" t="s">
@@ -2454,76 +2458,76 @@
       <c r="B36" s="33"/>
       <c r="C36" s="34"/>
       <c r="D36" s="26"/>
-      <c r="E36" s="154" t="s">
+      <c r="E36" s="250" t="s">
         <v>32</v>
       </c>
-      <c r="F36" s="138"/>
-      <c r="G36" s="138"/>
-      <c r="H36" s="138"/>
-      <c r="I36" s="139"/>
-      <c r="J36" s="143" t="str">
+      <c r="F36" s="140"/>
+      <c r="G36" s="140"/>
+      <c r="H36" s="140"/>
+      <c r="I36" s="141"/>
+      <c r="J36" s="239" t="str">
         <f>IF(SUM(J28:K34)=0, "", MROUND(SUM(J28:K34), 10))</f>
         <v/>
       </c>
-      <c r="K36" s="265"/>
+      <c r="K36" s="240"/>
     </row>
     <row r="37" spans="1:11">
-      <c r="A37" s="166" t="s">
+      <c r="A37" s="194" t="s">
         <v>33</v>
       </c>
-      <c r="B37" s="145"/>
-      <c r="C37" s="145"/>
-      <c r="D37" s="145"/>
-      <c r="E37" s="145"/>
-      <c r="F37" s="145"/>
-      <c r="G37" s="145"/>
-      <c r="H37" s="145"/>
-      <c r="I37" s="145"/>
-      <c r="J37" s="145"/>
-      <c r="K37" s="145"/>
+      <c r="B37" s="179"/>
+      <c r="C37" s="179"/>
+      <c r="D37" s="179"/>
+      <c r="E37" s="179"/>
+      <c r="F37" s="179"/>
+      <c r="G37" s="179"/>
+      <c r="H37" s="179"/>
+      <c r="I37" s="179"/>
+      <c r="J37" s="179"/>
+      <c r="K37" s="179"/>
     </row>
     <row r="38" spans="1:11">
-      <c r="A38" s="155" t="s">
+      <c r="A38" s="266" t="s">
         <v>34</v>
       </c>
-      <c r="B38" s="145"/>
-      <c r="C38" s="145"/>
-      <c r="D38" s="145"/>
-      <c r="E38" s="145"/>
-      <c r="F38" s="145"/>
-      <c r="G38" s="145"/>
-      <c r="H38" s="145"/>
-      <c r="I38" s="145"/>
-      <c r="J38" s="145"/>
-      <c r="K38" s="145"/>
+      <c r="B38" s="179"/>
+      <c r="C38" s="179"/>
+      <c r="D38" s="179"/>
+      <c r="E38" s="179"/>
+      <c r="F38" s="179"/>
+      <c r="G38" s="179"/>
+      <c r="H38" s="179"/>
+      <c r="I38" s="179"/>
+      <c r="J38" s="179"/>
+      <c r="K38" s="179"/>
     </row>
     <row r="39" spans="1:11">
-      <c r="A39" s="188" t="s">
+      <c r="A39" s="245" t="s">
         <v>35</v>
       </c>
-      <c r="B39" s="138"/>
-      <c r="C39" s="139"/>
+      <c r="B39" s="140"/>
+      <c r="C39" s="141"/>
       <c r="D39" s="35"/>
-      <c r="E39" s="136" t="s">
+      <c r="E39" s="135" t="s">
         <v>36</v>
       </c>
       <c r="F39" s="58"/>
       <c r="G39" s="51"/>
-      <c r="H39" s="153" t="s">
+      <c r="H39" s="258" t="s">
         <v>24</v>
       </c>
-      <c r="I39" s="138"/>
-      <c r="J39" s="138"/>
-      <c r="K39" s="139"/>
+      <c r="I39" s="140"/>
+      <c r="J39" s="140"/>
+      <c r="K39" s="141"/>
     </row>
     <row r="40" spans="1:11">
-      <c r="A40" s="173" t="s">
+      <c r="A40" s="241" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="173" t="s">
+      <c r="B40" s="241" t="s">
         <v>38</v>
       </c>
-      <c r="C40" s="269" t="s">
+      <c r="C40" s="270" t="s">
         <v>27</v>
       </c>
       <c r="D40" s="26"/>
@@ -2532,33 +2536,33 @@
       </c>
       <c r="F40" s="37"/>
       <c r="G40" s="38"/>
-      <c r="H40" s="156" t="s">
+      <c r="H40" s="234" t="s">
         <v>40</v>
       </c>
-      <c r="I40" s="156" t="s">
+      <c r="I40" s="234" t="s">
         <v>41</v>
       </c>
-      <c r="J40" s="156" t="s">
+      <c r="J40" s="234" t="s">
         <v>42</v>
       </c>
-      <c r="K40" s="156" t="s">
+      <c r="K40" s="234" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="41" spans="1:11">
-      <c r="A41" s="174"/>
-      <c r="B41" s="174"/>
-      <c r="C41" s="174"/>
+      <c r="A41" s="235"/>
+      <c r="B41" s="235"/>
+      <c r="C41" s="235"/>
       <c r="D41" s="26"/>
       <c r="E41" s="37" t="s">
         <v>44</v>
       </c>
       <c r="F41" s="37"/>
       <c r="G41" s="52"/>
-      <c r="H41" s="174"/>
-      <c r="I41" s="270"/>
-      <c r="J41" s="270"/>
-      <c r="K41" s="174"/>
+      <c r="H41" s="235"/>
+      <c r="I41" s="252"/>
+      <c r="J41" s="252"/>
+      <c r="K41" s="235"/>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" s="39"/>
@@ -2694,11 +2698,11 @@
       <c r="B45" s="43"/>
       <c r="C45" s="43"/>
       <c r="D45" s="26"/>
-      <c r="E45" s="164" t="s">
+      <c r="E45" s="272" t="s">
         <v>39</v>
       </c>
-      <c r="F45" s="145"/>
-      <c r="G45" s="165"/>
+      <c r="F45" s="179"/>
+      <c r="G45" s="273"/>
       <c r="H45" s="82"/>
       <c r="I45" s="83"/>
       <c r="J45" s="111" t="str" cm="1">
@@ -2816,9 +2820,9 @@
       <c r="B51" s="15"/>
       <c r="C51" s="15"/>
       <c r="D51" s="11"/>
-      <c r="E51" s="140"/>
-      <c r="F51" s="141"/>
-      <c r="G51" s="142"/>
+      <c r="E51" s="236"/>
+      <c r="F51" s="159"/>
+      <c r="G51" s="165"/>
       <c r="H51" s="82"/>
       <c r="I51" s="82"/>
       <c r="J51" s="104"/>
@@ -2853,58 +2857,58 @@
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
-      <c r="H53" s="169"/>
-      <c r="I53" s="138"/>
-      <c r="J53" s="139"/>
+      <c r="H53" s="154"/>
+      <c r="I53" s="140"/>
+      <c r="J53" s="141"/>
       <c r="K53" s="110" t="str">
         <f>IF(SUM(K42:K51)=0, "", MROUND(SUM(K42:K51), 10))</f>
         <v/>
       </c>
     </row>
     <row r="54" spans="1:11">
-      <c r="A54" s="181"/>
-      <c r="B54" s="138"/>
-      <c r="C54" s="138"/>
-      <c r="D54" s="138"/>
-      <c r="E54" s="138"/>
-      <c r="F54" s="138"/>
-      <c r="G54" s="138"/>
-      <c r="H54" s="138"/>
-      <c r="I54" s="138"/>
-      <c r="J54" s="138"/>
-      <c r="K54" s="138"/>
+      <c r="A54" s="275"/>
+      <c r="B54" s="140"/>
+      <c r="C54" s="140"/>
+      <c r="D54" s="140"/>
+      <c r="E54" s="140"/>
+      <c r="F54" s="140"/>
+      <c r="G54" s="140"/>
+      <c r="H54" s="140"/>
+      <c r="I54" s="140"/>
+      <c r="J54" s="140"/>
+      <c r="K54" s="140"/>
     </row>
     <row r="55" spans="1:11">
-      <c r="A55" s="151" t="s">
+      <c r="A55" s="264" t="s">
         <v>56</v>
       </c>
-      <c r="B55" s="141"/>
-      <c r="C55" s="141"/>
-      <c r="D55" s="141"/>
-      <c r="E55" s="141"/>
-      <c r="F55" s="141"/>
-      <c r="G55" s="141"/>
-      <c r="H55" s="141"/>
-      <c r="I55" s="141"/>
-      <c r="J55" s="141"/>
-      <c r="K55" s="141"/>
+      <c r="B55" s="159"/>
+      <c r="C55" s="159"/>
+      <c r="D55" s="159"/>
+      <c r="E55" s="159"/>
+      <c r="F55" s="159"/>
+      <c r="G55" s="159"/>
+      <c r="H55" s="159"/>
+      <c r="I55" s="159"/>
+      <c r="J55" s="159"/>
+      <c r="K55" s="159"/>
     </row>
     <row r="56" spans="1:11">
-      <c r="A56" s="137" t="s">
+      <c r="A56" s="269" t="s">
         <v>35</v>
       </c>
-      <c r="B56" s="138"/>
-      <c r="C56" s="139"/>
+      <c r="B56" s="140"/>
+      <c r="C56" s="141"/>
       <c r="D56" s="53"/>
-      <c r="E56" s="163" t="s">
+      <c r="E56" s="271" t="s">
         <v>57</v>
       </c>
-      <c r="F56" s="138"/>
-      <c r="G56" s="138"/>
-      <c r="H56" s="138"/>
-      <c r="I56" s="138"/>
-      <c r="J56" s="138"/>
-      <c r="K56" s="138"/>
+      <c r="F56" s="140"/>
+      <c r="G56" s="140"/>
+      <c r="H56" s="140"/>
+      <c r="I56" s="140"/>
+      <c r="J56" s="140"/>
+      <c r="K56" s="140"/>
     </row>
     <row r="57" spans="1:11">
       <c r="A57" s="6" t="s">
@@ -2930,46 +2934,46 @@
       <c r="I57" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="J57" s="192" t="s">
+      <c r="J57" s="231" t="s">
         <v>59</v>
       </c>
-      <c r="K57" s="162"/>
+      <c r="K57" s="232"/>
     </row>
     <row r="58" spans="1:11">
       <c r="A58" s="81"/>
       <c r="B58" s="75"/>
       <c r="C58" s="81"/>
       <c r="D58" s="91"/>
-      <c r="E58" s="190"/>
-      <c r="F58" s="264"/>
+      <c r="E58" s="227"/>
+      <c r="F58" s="249"/>
       <c r="G58" s="92"/>
       <c r="H58" s="103"/>
       <c r="I58" s="80"/>
-      <c r="J58" s="186"/>
-      <c r="K58" s="265"/>
+      <c r="J58" s="276"/>
+      <c r="K58" s="240"/>
     </row>
     <row r="59" spans="1:11">
       <c r="A59" s="81"/>
       <c r="B59" s="81"/>
       <c r="C59" s="81"/>
       <c r="D59" s="91"/>
-      <c r="E59" s="190"/>
-      <c r="F59" s="267"/>
+      <c r="E59" s="227"/>
+      <c r="F59" s="228"/>
       <c r="G59" s="92"/>
       <c r="H59" s="92"/>
       <c r="I59" s="84" t="s">
         <v>39</v>
       </c>
-      <c r="J59" s="187"/>
-      <c r="K59" s="271"/>
+      <c r="J59" s="277"/>
+      <c r="K59" s="278"/>
     </row>
     <row r="60" spans="1:11" hidden="1">
       <c r="A60" s="12"/>
       <c r="B60" s="12"/>
       <c r="C60" s="12"/>
       <c r="D60" s="17"/>
-      <c r="E60" s="148"/>
-      <c r="F60" s="148"/>
+      <c r="E60" s="262"/>
+      <c r="F60" s="262"/>
       <c r="G60" s="18" t="s">
         <v>39</v>
       </c>
@@ -2979,8 +2983,8 @@
       <c r="I60" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="J60" s="180"/>
-      <c r="K60" s="139"/>
+      <c r="J60" s="274"/>
+      <c r="K60" s="141"/>
     </row>
     <row r="61" spans="1:11">
       <c r="A61" s="1" t="s">
@@ -2989,10 +2993,10 @@
       <c r="B61" s="12"/>
       <c r="C61" s="94"/>
       <c r="D61" s="17"/>
-      <c r="E61" s="157" t="s">
+      <c r="E61" s="267" t="s">
         <v>31</v>
       </c>
-      <c r="F61" s="139"/>
+      <c r="F61" s="141"/>
       <c r="G61" s="93"/>
       <c r="H61" s="18" t="s">
         <v>39</v>
@@ -3000,24 +3004,24 @@
       <c r="I61" s="84" t="s">
         <v>39</v>
       </c>
-      <c r="J61" s="158" t="str">
+      <c r="J61" s="268" t="str">
         <f>IF(SUM(J58:K59)=0, "", MROUND(SUM(J58:K59), 10))</f>
         <v/>
       </c>
-      <c r="K61" s="264"/>
+      <c r="K61" s="249"/>
     </row>
     <row r="62" spans="1:11">
-      <c r="A62" s="140"/>
-      <c r="B62" s="141"/>
-      <c r="C62" s="141"/>
-      <c r="D62" s="141"/>
-      <c r="E62" s="141"/>
-      <c r="F62" s="141"/>
-      <c r="G62" s="141"/>
-      <c r="H62" s="141"/>
-      <c r="I62" s="141"/>
-      <c r="J62" s="141"/>
-      <c r="K62" s="142"/>
+      <c r="A62" s="236"/>
+      <c r="B62" s="159"/>
+      <c r="C62" s="159"/>
+      <c r="D62" s="159"/>
+      <c r="E62" s="159"/>
+      <c r="F62" s="159"/>
+      <c r="G62" s="159"/>
+      <c r="H62" s="159"/>
+      <c r="I62" s="159"/>
+      <c r="J62" s="159"/>
+      <c r="K62" s="165"/>
     </row>
     <row r="63" spans="1:11" ht="0.75" customHeight="1">
       <c r="A63" s="54"/>
@@ -3033,43 +3037,109 @@
       <c r="A64" s="65" t="s">
         <v>60</v>
       </c>
-      <c r="B64" s="144"/>
-      <c r="C64" s="144"/>
-      <c r="D64" s="144"/>
-      <c r="E64" s="144"/>
-      <c r="F64" s="144"/>
-      <c r="G64" s="144"/>
-      <c r="H64" s="144"/>
-      <c r="I64" s="144"/>
-      <c r="J64" s="144"/>
-      <c r="K64" s="144"/>
+      <c r="B64" s="259"/>
+      <c r="C64" s="259"/>
+      <c r="D64" s="259"/>
+      <c r="E64" s="259"/>
+      <c r="F64" s="259"/>
+      <c r="G64" s="259"/>
+      <c r="H64" s="259"/>
+      <c r="I64" s="259"/>
+      <c r="J64" s="259"/>
+      <c r="K64" s="259"/>
     </row>
     <row r="65" spans="2:11">
-      <c r="B65" s="144"/>
-      <c r="C65" s="144"/>
-      <c r="D65" s="144"/>
-      <c r="E65" s="144"/>
-      <c r="F65" s="144"/>
-      <c r="G65" s="144"/>
-      <c r="H65" s="144"/>
-      <c r="I65" s="144"/>
-      <c r="J65" s="144"/>
-      <c r="K65" s="144"/>
+      <c r="B65" s="259"/>
+      <c r="C65" s="259"/>
+      <c r="D65" s="259"/>
+      <c r="E65" s="259"/>
+      <c r="F65" s="259"/>
+      <c r="G65" s="259"/>
+      <c r="H65" s="259"/>
+      <c r="I65" s="259"/>
+      <c r="J65" s="259"/>
+      <c r="K65" s="259"/>
     </row>
     <row r="66" spans="2:11" ht="39" customHeight="1">
-      <c r="B66" s="144"/>
-      <c r="C66" s="144"/>
-      <c r="D66" s="144"/>
-      <c r="E66" s="144"/>
-      <c r="F66" s="144"/>
-      <c r="G66" s="144"/>
-      <c r="H66" s="144"/>
-      <c r="I66" s="144"/>
-      <c r="J66" s="144"/>
-      <c r="K66" s="144"/>
+      <c r="B66" s="259"/>
+      <c r="C66" s="259"/>
+      <c r="D66" s="259"/>
+      <c r="E66" s="259"/>
+      <c r="F66" s="259"/>
+      <c r="G66" s="259"/>
+      <c r="H66" s="259"/>
+      <c r="I66" s="259"/>
+      <c r="J66" s="259"/>
+      <c r="K66" s="259"/>
     </row>
   </sheetData>
   <mergeCells count="82">
+    <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A62:K62"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="E56:K56"/>
+    <mergeCell ref="E45:G45"/>
+    <mergeCell ref="H53:J53"/>
+    <mergeCell ref="J60:K60"/>
+    <mergeCell ref="A54:K54"/>
+    <mergeCell ref="J58:K58"/>
+    <mergeCell ref="J59:K59"/>
+    <mergeCell ref="B64:K66"/>
+    <mergeCell ref="E28:F28"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="A55:K55"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="E36:I36"/>
+    <mergeCell ref="A38:K38"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="I40:I41"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="J61:K61"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="C7:I7"/>
+    <mergeCell ref="H40:H41"/>
+    <mergeCell ref="J40:J41"/>
+    <mergeCell ref="E29:F29"/>
+    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="E31:F31"/>
+    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A23:K23"/>
+    <mergeCell ref="E32:F32"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="E34:F34"/>
+    <mergeCell ref="H39:K39"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="C5:G5"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="E33:F33"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="E35:F35"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="A25:K25"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="A24:K24"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="H13:K13"/>
     <mergeCell ref="B13:G13"/>
     <mergeCell ref="A8:K8"/>
@@ -3086,72 +3156,6 @@
     <mergeCell ref="H19:I19"/>
     <mergeCell ref="C18:E18"/>
     <mergeCell ref="E27:F27"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="A24:K24"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="C5:G5"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="E33:F33"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="E35:F35"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="A25:K25"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="C7:I7"/>
-    <mergeCell ref="H40:H41"/>
-    <mergeCell ref="J40:J41"/>
-    <mergeCell ref="E29:F29"/>
-    <mergeCell ref="A37:K37"/>
-    <mergeCell ref="E31:F31"/>
-    <mergeCell ref="A14:K14"/>
-    <mergeCell ref="A23:K23"/>
-    <mergeCell ref="E32:F32"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="E34:F34"/>
-    <mergeCell ref="H39:K39"/>
-    <mergeCell ref="B64:K66"/>
-    <mergeCell ref="E28:F28"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="E60:F60"/>
-    <mergeCell ref="E30:F30"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="A55:K55"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="E36:I36"/>
-    <mergeCell ref="A38:K38"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="I40:I41"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="J61:K61"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="A56:C56"/>
-    <mergeCell ref="A62:K62"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="E56:K56"/>
-    <mergeCell ref="E45:G45"/>
-    <mergeCell ref="H53:J53"/>
-    <mergeCell ref="J60:K60"/>
-    <mergeCell ref="A54:K54"/>
-    <mergeCell ref="J58:K58"/>
-    <mergeCell ref="J59:K59"/>
   </mergeCells>
   <conditionalFormatting sqref="G28:G33">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -3169,7 +3173,7 @@
   <sheetPr codeName="Sheet5">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AA71"/>
+  <dimension ref="A1:AA72"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
@@ -3189,270 +3193,270 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13">
-      <c r="A1" s="224" t="s">
+      <c r="A1" s="175" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="141"/>
-      <c r="C1" s="141"/>
-      <c r="D1" s="141"/>
-      <c r="E1" s="141"/>
-      <c r="F1" s="141"/>
-      <c r="G1" s="141"/>
-      <c r="H1" s="141"/>
-      <c r="I1" s="141"/>
-      <c r="J1" s="141"/>
-      <c r="K1" s="141"/>
-      <c r="L1" s="141"/>
-      <c r="M1" s="141"/>
+      <c r="B1" s="159"/>
+      <c r="C1" s="159"/>
+      <c r="D1" s="159"/>
+      <c r="E1" s="159"/>
+      <c r="F1" s="159"/>
+      <c r="G1" s="159"/>
+      <c r="H1" s="159"/>
+      <c r="I1" s="159"/>
+      <c r="J1" s="159"/>
+      <c r="K1" s="159"/>
+      <c r="L1" s="159"/>
+      <c r="M1" s="159"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A2" s="177" t="s">
+      <c r="A2" s="168" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="178"/>
-      <c r="C2" s="178"/>
-      <c r="D2" s="178"/>
-      <c r="E2" s="178"/>
-      <c r="F2" s="178"/>
-      <c r="G2" s="178"/>
-      <c r="H2" s="178"/>
-      <c r="I2" s="178"/>
-      <c r="J2" s="178"/>
-      <c r="K2" s="178"/>
-      <c r="L2" s="178"/>
-      <c r="M2" s="178"/>
+      <c r="B2" s="138"/>
+      <c r="C2" s="138"/>
+      <c r="D2" s="138"/>
+      <c r="E2" s="138"/>
+      <c r="F2" s="138"/>
+      <c r="G2" s="138"/>
+      <c r="H2" s="138"/>
+      <c r="I2" s="138"/>
+      <c r="J2" s="138"/>
+      <c r="K2" s="138"/>
+      <c r="L2" s="138"/>
+      <c r="M2" s="138"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="197" t="s">
+      <c r="A3" s="169" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="217"/>
-      <c r="C3" s="217"/>
-      <c r="D3" s="218"/>
-      <c r="E3" s="216" t="s">
+      <c r="B3" s="170"/>
+      <c r="C3" s="170"/>
+      <c r="D3" s="171"/>
+      <c r="E3" s="142" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="195" t="s">
+      <c r="F3" s="162" t="s">
         <v>64</v>
       </c>
-      <c r="G3" s="196"/>
-      <c r="H3" s="196"/>
-      <c r="I3" s="196"/>
-      <c r="J3" s="196"/>
-      <c r="K3" s="196"/>
-      <c r="L3" s="197"/>
-      <c r="M3" s="195" t="s">
+      <c r="G3" s="180"/>
+      <c r="H3" s="180"/>
+      <c r="I3" s="180"/>
+      <c r="J3" s="180"/>
+      <c r="K3" s="180"/>
+      <c r="L3" s="169"/>
+      <c r="M3" s="162" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="13.5" customHeight="1">
-      <c r="A4" s="220"/>
-      <c r="B4" s="220"/>
-      <c r="C4" s="220"/>
-      <c r="D4" s="221"/>
-      <c r="E4" s="246"/>
-      <c r="F4" s="195" t="s">
+      <c r="A4" s="172"/>
+      <c r="B4" s="172"/>
+      <c r="C4" s="172"/>
+      <c r="D4" s="173"/>
+      <c r="E4" s="143"/>
+      <c r="F4" s="162" t="s">
         <v>65</v>
       </c>
-      <c r="G4" s="197"/>
-      <c r="H4" s="195" t="s">
+      <c r="G4" s="169"/>
+      <c r="H4" s="162" t="s">
         <v>66</v>
       </c>
-      <c r="I4" s="196"/>
-      <c r="J4" s="197"/>
-      <c r="K4" s="135" t="s">
+      <c r="I4" s="180"/>
+      <c r="J4" s="169"/>
+      <c r="K4" s="134" t="s">
         <v>67</v>
       </c>
-      <c r="L4" s="135" t="s">
+      <c r="L4" s="134" t="s">
         <v>68</v>
       </c>
-      <c r="M4" s="219"/>
+      <c r="M4" s="163"/>
     </row>
     <row r="5" spans="1:13">
-      <c r="A5" s="249"/>
-      <c r="B5" s="138"/>
-      <c r="C5" s="138"/>
-      <c r="D5" s="139"/>
+      <c r="A5" s="183"/>
+      <c r="B5" s="140"/>
+      <c r="C5" s="140"/>
+      <c r="D5" s="141"/>
       <c r="E5" s="28"/>
-      <c r="F5" s="191"/>
-      <c r="G5" s="182"/>
-      <c r="H5" s="191"/>
-      <c r="I5" s="233"/>
-      <c r="J5" s="182"/>
+      <c r="F5" s="223"/>
+      <c r="G5" s="205"/>
+      <c r="H5" s="223"/>
+      <c r="I5" s="144"/>
+      <c r="J5" s="205"/>
       <c r="K5" s="28"/>
       <c r="L5" s="28"/>
       <c r="M5" s="50"/>
     </row>
     <row r="6" spans="1:13">
-      <c r="A6" s="206"/>
-      <c r="B6" s="138"/>
-      <c r="C6" s="138"/>
-      <c r="D6" s="139"/>
+      <c r="A6" s="139"/>
+      <c r="B6" s="140"/>
+      <c r="C6" s="140"/>
+      <c r="D6" s="141"/>
       <c r="E6" s="56"/>
-      <c r="F6" s="198"/>
-      <c r="G6" s="199"/>
-      <c r="H6" s="198"/>
-      <c r="I6" s="234"/>
-      <c r="J6" s="199"/>
+      <c r="F6" s="155"/>
+      <c r="G6" s="157"/>
+      <c r="H6" s="155"/>
+      <c r="I6" s="156"/>
+      <c r="J6" s="157"/>
       <c r="K6" s="56"/>
       <c r="L6" s="56"/>
-      <c r="M6" s="134"/>
+      <c r="M6" s="133"/>
     </row>
     <row r="7" spans="1:13">
-      <c r="A7" s="206"/>
-      <c r="B7" s="138"/>
-      <c r="C7" s="138"/>
-      <c r="D7" s="139"/>
+      <c r="A7" s="139"/>
+      <c r="B7" s="140"/>
+      <c r="C7" s="140"/>
+      <c r="D7" s="141"/>
       <c r="E7" s="56"/>
-      <c r="F7" s="198"/>
-      <c r="G7" s="199"/>
-      <c r="H7" s="198"/>
-      <c r="I7" s="234"/>
-      <c r="J7" s="199"/>
+      <c r="F7" s="155"/>
+      <c r="G7" s="157"/>
+      <c r="H7" s="155"/>
+      <c r="I7" s="156"/>
+      <c r="J7" s="157"/>
       <c r="K7" s="56"/>
       <c r="L7" s="56"/>
-      <c r="M7" s="134"/>
+      <c r="M7" s="133"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A8" s="232" t="s">
+      <c r="A8" s="193" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="178"/>
-      <c r="C8" s="178"/>
-      <c r="D8" s="178"/>
-      <c r="E8" s="178"/>
-      <c r="F8" s="178"/>
-      <c r="G8" s="178"/>
-      <c r="H8" s="178"/>
-      <c r="I8" s="178"/>
-      <c r="J8" s="178"/>
-      <c r="K8" s="178"/>
-      <c r="L8" s="178"/>
+      <c r="B8" s="138"/>
+      <c r="C8" s="138"/>
+      <c r="D8" s="138"/>
+      <c r="E8" s="138"/>
+      <c r="F8" s="138"/>
+      <c r="G8" s="138"/>
+      <c r="H8" s="138"/>
+      <c r="I8" s="138"/>
+      <c r="J8" s="138"/>
+      <c r="K8" s="138"/>
+      <c r="L8" s="138"/>
       <c r="M8" s="51"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A9" s="210" t="s">
+      <c r="A9" s="145" t="s">
         <v>70</v>
       </c>
-      <c r="B9" s="138"/>
-      <c r="C9" s="138"/>
-      <c r="D9" s="138"/>
-      <c r="E9" s="138"/>
-      <c r="F9" s="138"/>
-      <c r="G9" s="138"/>
-      <c r="H9" s="138"/>
-      <c r="I9" s="138"/>
-      <c r="J9" s="138"/>
-      <c r="K9" s="138"/>
-      <c r="L9" s="138"/>
-      <c r="M9" s="138"/>
+      <c r="B9" s="140"/>
+      <c r="C9" s="140"/>
+      <c r="D9" s="140"/>
+      <c r="E9" s="140"/>
+      <c r="F9" s="140"/>
+      <c r="G9" s="140"/>
+      <c r="H9" s="140"/>
+      <c r="I9" s="140"/>
+      <c r="J9" s="140"/>
+      <c r="K9" s="140"/>
+      <c r="L9" s="140"/>
+      <c r="M9" s="140"/>
     </row>
     <row r="10" spans="1:13">
-      <c r="A10" s="197" t="s">
+      <c r="A10" s="169" t="s">
         <v>63</v>
       </c>
-      <c r="B10" s="217"/>
-      <c r="C10" s="217"/>
-      <c r="D10" s="218"/>
-      <c r="E10" s="216" t="s">
+      <c r="B10" s="170"/>
+      <c r="C10" s="170"/>
+      <c r="D10" s="171"/>
+      <c r="E10" s="142" t="s">
         <v>115</v>
       </c>
-      <c r="F10" s="195" t="s">
+      <c r="F10" s="162" t="s">
         <v>64</v>
       </c>
-      <c r="G10" s="196"/>
-      <c r="H10" s="196"/>
-      <c r="I10" s="196"/>
-      <c r="J10" s="196"/>
-      <c r="K10" s="196"/>
-      <c r="L10" s="197"/>
-      <c r="M10" s="195" t="s">
+      <c r="G10" s="180"/>
+      <c r="H10" s="180"/>
+      <c r="I10" s="180"/>
+      <c r="J10" s="180"/>
+      <c r="K10" s="180"/>
+      <c r="L10" s="169"/>
+      <c r="M10" s="162" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.5" customHeight="1">
-      <c r="A11" s="220"/>
-      <c r="B11" s="220"/>
-      <c r="C11" s="220"/>
-      <c r="D11" s="221"/>
-      <c r="E11" s="246"/>
-      <c r="F11" s="195" t="s">
+      <c r="A11" s="172"/>
+      <c r="B11" s="172"/>
+      <c r="C11" s="172"/>
+      <c r="D11" s="173"/>
+      <c r="E11" s="143"/>
+      <c r="F11" s="162" t="s">
         <v>65</v>
       </c>
-      <c r="G11" s="197"/>
-      <c r="H11" s="195" t="s">
+      <c r="G11" s="169"/>
+      <c r="H11" s="162" t="s">
         <v>66</v>
       </c>
-      <c r="I11" s="196"/>
-      <c r="J11" s="197"/>
-      <c r="K11" s="135" t="s">
+      <c r="I11" s="180"/>
+      <c r="J11" s="169"/>
+      <c r="K11" s="134" t="s">
         <v>67</v>
       </c>
-      <c r="L11" s="135" t="s">
+      <c r="L11" s="134" t="s">
         <v>68</v>
       </c>
-      <c r="M11" s="219"/>
+      <c r="M11" s="163"/>
     </row>
     <row r="12" spans="1:13" ht="12" customHeight="1">
-      <c r="A12" s="206"/>
-      <c r="B12" s="138"/>
-      <c r="C12" s="138"/>
-      <c r="D12" s="139"/>
+      <c r="A12" s="139"/>
+      <c r="B12" s="140"/>
+      <c r="C12" s="140"/>
+      <c r="D12" s="141"/>
       <c r="E12" s="56"/>
-      <c r="F12" s="198"/>
-      <c r="G12" s="199"/>
-      <c r="H12" s="198"/>
-      <c r="I12" s="234"/>
-      <c r="J12" s="199"/>
+      <c r="F12" s="155"/>
+      <c r="G12" s="157"/>
+      <c r="H12" s="155"/>
+      <c r="I12" s="156"/>
+      <c r="J12" s="157"/>
       <c r="K12" s="56"/>
       <c r="L12" s="56"/>
       <c r="M12" s="50"/>
     </row>
     <row r="13" spans="1:13">
-      <c r="A13" s="206"/>
-      <c r="B13" s="138"/>
-      <c r="C13" s="138"/>
-      <c r="D13" s="139"/>
+      <c r="A13" s="139"/>
+      <c r="B13" s="140"/>
+      <c r="C13" s="140"/>
+      <c r="D13" s="141"/>
       <c r="E13" s="56"/>
-      <c r="F13" s="198"/>
-      <c r="G13" s="199"/>
-      <c r="H13" s="198"/>
-      <c r="I13" s="234"/>
-      <c r="J13" s="199"/>
+      <c r="F13" s="155"/>
+      <c r="G13" s="157"/>
+      <c r="H13" s="155"/>
+      <c r="I13" s="156"/>
+      <c r="J13" s="157"/>
       <c r="K13" s="56"/>
       <c r="L13" s="56"/>
-      <c r="M13" s="134"/>
+      <c r="M13" s="133"/>
     </row>
     <row r="14" spans="1:13" ht="12" customHeight="1">
-      <c r="A14" s="206"/>
-      <c r="B14" s="138"/>
-      <c r="C14" s="138"/>
-      <c r="D14" s="139"/>
+      <c r="A14" s="139"/>
+      <c r="B14" s="140"/>
+      <c r="C14" s="140"/>
+      <c r="D14" s="141"/>
       <c r="E14" s="56"/>
-      <c r="F14" s="198"/>
-      <c r="G14" s="199"/>
-      <c r="H14" s="198"/>
-      <c r="I14" s="234"/>
-      <c r="J14" s="199"/>
+      <c r="F14" s="155"/>
+      <c r="G14" s="157"/>
+      <c r="H14" s="155"/>
+      <c r="I14" s="156"/>
+      <c r="J14" s="157"/>
       <c r="K14" s="56"/>
       <c r="L14" s="56"/>
-      <c r="M14" s="134"/>
+      <c r="M14" s="133"/>
     </row>
     <row r="15" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A15" s="234" t="s">
+      <c r="A15" s="156" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="138"/>
-      <c r="C15" s="138"/>
-      <c r="D15" s="138"/>
-      <c r="E15" s="138"/>
-      <c r="F15" s="138"/>
-      <c r="G15" s="138"/>
-      <c r="H15" s="138"/>
-      <c r="I15" s="138"/>
-      <c r="J15" s="138"/>
-      <c r="K15" s="138"/>
-      <c r="L15" s="138"/>
+      <c r="B15" s="140"/>
+      <c r="C15" s="140"/>
+      <c r="D15" s="140"/>
+      <c r="E15" s="140"/>
+      <c r="F15" s="140"/>
+      <c r="G15" s="140"/>
+      <c r="H15" s="140"/>
+      <c r="I15" s="140"/>
+      <c r="J15" s="140"/>
+      <c r="K15" s="140"/>
+      <c r="L15" s="140"/>
       <c r="M15" s="58"/>
     </row>
     <row r="16" spans="1:13" ht="5.25" customHeight="1">
@@ -3471,258 +3475,258 @@
       <c r="M16" s="21"/>
     </row>
     <row r="17" spans="1:13" ht="15" customHeight="1">
-      <c r="A17" s="224" t="s">
+      <c r="A17" s="175" t="s">
         <v>71</v>
       </c>
-      <c r="B17" s="141"/>
-      <c r="C17" s="141"/>
-      <c r="D17" s="141"/>
-      <c r="E17" s="141"/>
-      <c r="F17" s="141"/>
-      <c r="G17" s="141"/>
-      <c r="H17" s="141"/>
-      <c r="I17" s="141"/>
-      <c r="J17" s="141"/>
-      <c r="K17" s="141"/>
-      <c r="L17" s="141"/>
-      <c r="M17" s="141"/>
+      <c r="B17" s="159"/>
+      <c r="C17" s="159"/>
+      <c r="D17" s="159"/>
+      <c r="E17" s="159"/>
+      <c r="F17" s="159"/>
+      <c r="G17" s="159"/>
+      <c r="H17" s="159"/>
+      <c r="I17" s="159"/>
+      <c r="J17" s="159"/>
+      <c r="K17" s="159"/>
+      <c r="L17" s="159"/>
+      <c r="M17" s="159"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A18" s="210" t="s">
+      <c r="A18" s="145" t="s">
         <v>62</v>
       </c>
-      <c r="B18" s="138"/>
-      <c r="C18" s="138"/>
-      <c r="D18" s="138"/>
-      <c r="E18" s="138"/>
-      <c r="F18" s="138"/>
-      <c r="G18" s="138"/>
-      <c r="H18" s="138"/>
-      <c r="I18" s="138"/>
-      <c r="J18" s="138"/>
-      <c r="K18" s="138"/>
-      <c r="L18" s="138"/>
-      <c r="M18" s="138"/>
+      <c r="B18" s="140"/>
+      <c r="C18" s="140"/>
+      <c r="D18" s="140"/>
+      <c r="E18" s="140"/>
+      <c r="F18" s="140"/>
+      <c r="G18" s="140"/>
+      <c r="H18" s="140"/>
+      <c r="I18" s="140"/>
+      <c r="J18" s="140"/>
+      <c r="K18" s="140"/>
+      <c r="L18" s="140"/>
+      <c r="M18" s="140"/>
     </row>
     <row r="19" spans="1:13" ht="8.25" customHeight="1">
-      <c r="A19" s="197" t="s">
+      <c r="A19" s="169" t="s">
         <v>63</v>
       </c>
-      <c r="B19" s="217"/>
-      <c r="C19" s="217"/>
-      <c r="D19" s="218"/>
-      <c r="E19" s="216" t="s">
+      <c r="B19" s="170"/>
+      <c r="C19" s="170"/>
+      <c r="D19" s="171"/>
+      <c r="E19" s="142" t="s">
         <v>72</v>
       </c>
-      <c r="F19" s="217"/>
-      <c r="G19" s="218"/>
-      <c r="H19" s="251" t="s">
+      <c r="F19" s="170"/>
+      <c r="G19" s="171"/>
+      <c r="H19" s="146" t="s">
         <v>73</v>
       </c>
-      <c r="I19" s="225"/>
-      <c r="J19" s="252"/>
-      <c r="K19" s="216" t="s">
+      <c r="I19" s="147"/>
+      <c r="J19" s="148"/>
+      <c r="K19" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="L19" s="218"/>
-      <c r="M19" s="195" t="s">
+      <c r="L19" s="171"/>
+      <c r="M19" s="162" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="6.75" customHeight="1">
-      <c r="A20" s="220"/>
-      <c r="B20" s="220"/>
-      <c r="C20" s="220"/>
-      <c r="D20" s="221"/>
-      <c r="E20" s="219"/>
-      <c r="F20" s="220"/>
-      <c r="G20" s="221"/>
-      <c r="H20" s="253"/>
-      <c r="I20" s="254"/>
-      <c r="J20" s="255"/>
-      <c r="K20" s="219"/>
-      <c r="L20" s="221"/>
-      <c r="M20" s="219"/>
+      <c r="A20" s="172"/>
+      <c r="B20" s="172"/>
+      <c r="C20" s="172"/>
+      <c r="D20" s="173"/>
+      <c r="E20" s="163"/>
+      <c r="F20" s="172"/>
+      <c r="G20" s="173"/>
+      <c r="H20" s="149"/>
+      <c r="I20" s="150"/>
+      <c r="J20" s="151"/>
+      <c r="K20" s="163"/>
+      <c r="L20" s="173"/>
+      <c r="M20" s="163"/>
     </row>
     <row r="21" spans="1:13" ht="15.6" customHeight="1">
-      <c r="A21" s="206"/>
-      <c r="B21" s="138"/>
-      <c r="C21" s="138"/>
-      <c r="D21" s="139"/>
-      <c r="E21" s="211"/>
-      <c r="F21" s="138"/>
-      <c r="G21" s="139"/>
-      <c r="H21" s="256"/>
-      <c r="I21" s="257"/>
-      <c r="J21" s="169"/>
-      <c r="K21" s="211"/>
-      <c r="L21" s="139"/>
+      <c r="A21" s="139"/>
+      <c r="B21" s="140"/>
+      <c r="C21" s="140"/>
+      <c r="D21" s="141"/>
+      <c r="E21" s="160"/>
+      <c r="F21" s="140"/>
+      <c r="G21" s="141"/>
+      <c r="H21" s="152"/>
+      <c r="I21" s="153"/>
+      <c r="J21" s="154"/>
+      <c r="K21" s="160"/>
+      <c r="L21" s="141"/>
       <c r="M21" s="50"/>
     </row>
     <row r="22" spans="1:13" ht="16.5" customHeight="1">
-      <c r="A22" s="206"/>
-      <c r="B22" s="138"/>
-      <c r="C22" s="138"/>
-      <c r="D22" s="139"/>
-      <c r="E22" s="211"/>
-      <c r="F22" s="138"/>
-      <c r="G22" s="139"/>
-      <c r="H22" s="256"/>
-      <c r="I22" s="257"/>
-      <c r="J22" s="169"/>
-      <c r="K22" s="211"/>
-      <c r="L22" s="139"/>
-      <c r="M22" s="134"/>
+      <c r="A22" s="139"/>
+      <c r="B22" s="140"/>
+      <c r="C22" s="140"/>
+      <c r="D22" s="141"/>
+      <c r="E22" s="160"/>
+      <c r="F22" s="140"/>
+      <c r="G22" s="141"/>
+      <c r="H22" s="152"/>
+      <c r="I22" s="153"/>
+      <c r="J22" s="154"/>
+      <c r="K22" s="160"/>
+      <c r="L22" s="141"/>
+      <c r="M22" s="133"/>
     </row>
     <row r="23" spans="1:13" ht="13.5" customHeight="1">
-      <c r="A23" s="206"/>
-      <c r="B23" s="138"/>
-      <c r="C23" s="138"/>
-      <c r="D23" s="139"/>
-      <c r="E23" s="229"/>
-      <c r="F23" s="141"/>
-      <c r="G23" s="142"/>
+      <c r="A23" s="139"/>
+      <c r="B23" s="140"/>
+      <c r="C23" s="140"/>
+      <c r="D23" s="141"/>
+      <c r="E23" s="164"/>
+      <c r="F23" s="159"/>
+      <c r="G23" s="165"/>
       <c r="H23" s="66"/>
       <c r="I23" s="57"/>
       <c r="J23" s="57"/>
-      <c r="K23" s="229"/>
-      <c r="L23" s="142"/>
-      <c r="M23" s="134"/>
+      <c r="K23" s="164"/>
+      <c r="L23" s="165"/>
+      <c r="M23" s="133"/>
     </row>
     <row r="24" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A24" s="232" t="s">
+      <c r="A24" s="193" t="s">
         <v>69</v>
       </c>
-      <c r="B24" s="178"/>
-      <c r="C24" s="178"/>
-      <c r="D24" s="178"/>
-      <c r="E24" s="178"/>
-      <c r="F24" s="178"/>
-      <c r="G24" s="178"/>
-      <c r="H24" s="178"/>
-      <c r="I24" s="178"/>
-      <c r="J24" s="178"/>
-      <c r="K24" s="178"/>
-      <c r="L24" s="178"/>
+      <c r="B24" s="138"/>
+      <c r="C24" s="138"/>
+      <c r="D24" s="138"/>
+      <c r="E24" s="138"/>
+      <c r="F24" s="138"/>
+      <c r="G24" s="138"/>
+      <c r="H24" s="138"/>
+      <c r="I24" s="138"/>
+      <c r="J24" s="138"/>
+      <c r="K24" s="138"/>
+      <c r="L24" s="138"/>
       <c r="M24" s="51"/>
     </row>
     <row r="25" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A25" s="210" t="s">
+      <c r="A25" s="145" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="138"/>
-      <c r="C25" s="138"/>
-      <c r="D25" s="138"/>
-      <c r="E25" s="138"/>
-      <c r="F25" s="138"/>
-      <c r="G25" s="138"/>
-      <c r="H25" s="138"/>
-      <c r="I25" s="138"/>
-      <c r="J25" s="138"/>
-      <c r="K25" s="138"/>
-      <c r="L25" s="138"/>
-      <c r="M25" s="138"/>
+      <c r="B25" s="140"/>
+      <c r="C25" s="140"/>
+      <c r="D25" s="140"/>
+      <c r="E25" s="140"/>
+      <c r="F25" s="140"/>
+      <c r="G25" s="140"/>
+      <c r="H25" s="140"/>
+      <c r="I25" s="140"/>
+      <c r="J25" s="140"/>
+      <c r="K25" s="140"/>
+      <c r="L25" s="140"/>
+      <c r="M25" s="140"/>
     </row>
     <row r="26" spans="1:13" ht="6.75" customHeight="1">
-      <c r="A26" s="197" t="s">
+      <c r="A26" s="169" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="217"/>
-      <c r="C26" s="217"/>
-      <c r="D26" s="218"/>
-      <c r="E26" s="216" t="s">
+      <c r="B26" s="170"/>
+      <c r="C26" s="170"/>
+      <c r="D26" s="171"/>
+      <c r="E26" s="142" t="s">
         <v>72</v>
       </c>
-      <c r="F26" s="217"/>
-      <c r="G26" s="218"/>
-      <c r="H26" s="251" t="s">
+      <c r="F26" s="170"/>
+      <c r="G26" s="171"/>
+      <c r="H26" s="146" t="s">
         <v>116</v>
       </c>
-      <c r="I26" s="225"/>
-      <c r="J26" s="252"/>
-      <c r="K26" s="216" t="s">
+      <c r="I26" s="147"/>
+      <c r="J26" s="148"/>
+      <c r="K26" s="142" t="s">
         <v>74</v>
       </c>
-      <c r="L26" s="218"/>
-      <c r="M26" s="195" t="s">
+      <c r="L26" s="171"/>
+      <c r="M26" s="162" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="27" spans="1:13" ht="9" customHeight="1">
-      <c r="A27" s="220"/>
-      <c r="B27" s="220"/>
-      <c r="C27" s="220"/>
-      <c r="D27" s="221"/>
-      <c r="E27" s="219"/>
-      <c r="F27" s="220"/>
-      <c r="G27" s="221"/>
-      <c r="H27" s="253"/>
-      <c r="I27" s="254"/>
-      <c r="J27" s="255"/>
-      <c r="K27" s="219"/>
-      <c r="L27" s="221"/>
-      <c r="M27" s="219"/>
+      <c r="A27" s="172"/>
+      <c r="B27" s="172"/>
+      <c r="C27" s="172"/>
+      <c r="D27" s="173"/>
+      <c r="E27" s="163"/>
+      <c r="F27" s="172"/>
+      <c r="G27" s="173"/>
+      <c r="H27" s="149"/>
+      <c r="I27" s="150"/>
+      <c r="J27" s="151"/>
+      <c r="K27" s="163"/>
+      <c r="L27" s="173"/>
+      <c r="M27" s="163"/>
     </row>
     <row r="28" spans="1:13">
-      <c r="A28" s="206"/>
-      <c r="B28" s="138"/>
-      <c r="C28" s="138"/>
-      <c r="D28" s="139"/>
-      <c r="E28" s="211"/>
-      <c r="F28" s="138"/>
-      <c r="G28" s="139"/>
-      <c r="H28" s="256"/>
-      <c r="I28" s="257"/>
-      <c r="J28" s="169"/>
-      <c r="K28" s="211"/>
-      <c r="L28" s="139"/>
+      <c r="A28" s="139"/>
+      <c r="B28" s="140"/>
+      <c r="C28" s="140"/>
+      <c r="D28" s="141"/>
+      <c r="E28" s="160"/>
+      <c r="F28" s="140"/>
+      <c r="G28" s="141"/>
+      <c r="H28" s="152"/>
+      <c r="I28" s="153"/>
+      <c r="J28" s="154"/>
+      <c r="K28" s="160"/>
+      <c r="L28" s="141"/>
       <c r="M28" s="50"/>
     </row>
     <row r="29" spans="1:13">
-      <c r="A29" s="206"/>
-      <c r="B29" s="138"/>
-      <c r="C29" s="138"/>
-      <c r="D29" s="139"/>
-      <c r="E29" s="211"/>
-      <c r="F29" s="138"/>
-      <c r="G29" s="139"/>
+      <c r="A29" s="139"/>
+      <c r="B29" s="140"/>
+      <c r="C29" s="140"/>
+      <c r="D29" s="141"/>
+      <c r="E29" s="160"/>
+      <c r="F29" s="140"/>
+      <c r="G29" s="141"/>
       <c r="H29" s="105"/>
       <c r="I29" s="58"/>
       <c r="J29" s="58"/>
-      <c r="K29" s="211"/>
-      <c r="L29" s="139"/>
-      <c r="M29" s="134"/>
+      <c r="K29" s="160"/>
+      <c r="L29" s="141"/>
+      <c r="M29" s="133"/>
     </row>
     <row r="30" spans="1:13">
-      <c r="A30" s="206"/>
-      <c r="B30" s="138"/>
-      <c r="C30" s="138"/>
-      <c r="D30" s="139"/>
-      <c r="E30" s="211"/>
-      <c r="F30" s="138"/>
-      <c r="G30" s="139"/>
+      <c r="A30" s="139"/>
+      <c r="B30" s="140"/>
+      <c r="C30" s="140"/>
+      <c r="D30" s="141"/>
+      <c r="E30" s="160"/>
+      <c r="F30" s="140"/>
+      <c r="G30" s="141"/>
       <c r="H30" s="66"/>
       <c r="I30" s="57"/>
       <c r="J30" s="57"/>
-      <c r="K30" s="211"/>
-      <c r="L30" s="139"/>
-      <c r="M30" s="134"/>
+      <c r="K30" s="160"/>
+      <c r="L30" s="141"/>
+      <c r="M30" s="133"/>
     </row>
     <row r="31" spans="1:13" ht="15.75" customHeight="1">
-      <c r="A31" s="182" t="s">
+      <c r="A31" s="205" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="138"/>
-      <c r="C31" s="138"/>
-      <c r="D31" s="138"/>
-      <c r="E31" s="138"/>
-      <c r="F31" s="138"/>
-      <c r="G31" s="138"/>
-      <c r="H31" s="138"/>
-      <c r="I31" s="138"/>
-      <c r="J31" s="138"/>
-      <c r="K31" s="138"/>
-      <c r="L31" s="139"/>
+      <c r="B31" s="140"/>
+      <c r="C31" s="140"/>
+      <c r="D31" s="140"/>
+      <c r="E31" s="140"/>
+      <c r="F31" s="140"/>
+      <c r="G31" s="140"/>
+      <c r="H31" s="140"/>
+      <c r="I31" s="140"/>
+      <c r="J31" s="140"/>
+      <c r="K31" s="140"/>
+      <c r="L31" s="141"/>
       <c r="M31" s="58"/>
     </row>
     <row r="32" spans="1:13">
@@ -3741,55 +3745,55 @@
       <c r="M32" s="21"/>
     </row>
     <row r="33" spans="1:14" ht="15.6" customHeight="1">
-      <c r="A33" s="247" t="s">
+      <c r="A33" s="181" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="145"/>
-      <c r="C33" s="145"/>
-      <c r="D33" s="145"/>
-      <c r="E33" s="145"/>
-      <c r="F33" s="145"/>
-      <c r="G33" s="145"/>
-      <c r="H33" s="145"/>
-      <c r="I33" s="145"/>
-      <c r="J33" s="145"/>
-      <c r="K33" s="145"/>
-      <c r="L33" s="145"/>
-      <c r="M33" s="145"/>
+      <c r="B33" s="179"/>
+      <c r="C33" s="179"/>
+      <c r="D33" s="179"/>
+      <c r="E33" s="179"/>
+      <c r="F33" s="179"/>
+      <c r="G33" s="179"/>
+      <c r="H33" s="179"/>
+      <c r="I33" s="179"/>
+      <c r="J33" s="179"/>
+      <c r="K33" s="179"/>
+      <c r="L33" s="179"/>
+      <c r="M33" s="179"/>
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1">
-      <c r="A34" s="214" t="s">
+      <c r="A34" s="176" t="s">
         <v>112</v>
       </c>
-      <c r="B34" s="215"/>
-      <c r="C34" s="215"/>
-      <c r="D34" s="215"/>
-      <c r="E34" s="215"/>
-      <c r="F34" s="215"/>
-      <c r="G34" s="215"/>
-      <c r="H34" s="215"/>
-      <c r="I34" s="215"/>
-      <c r="J34" s="215"/>
-      <c r="K34" s="215"/>
-      <c r="L34" s="215"/>
-      <c r="M34" s="215"/>
+      <c r="B34" s="177"/>
+      <c r="C34" s="177"/>
+      <c r="D34" s="177"/>
+      <c r="E34" s="177"/>
+      <c r="F34" s="177"/>
+      <c r="G34" s="177"/>
+      <c r="H34" s="177"/>
+      <c r="I34" s="177"/>
+      <c r="J34" s="177"/>
+      <c r="K34" s="177"/>
+      <c r="L34" s="177"/>
+      <c r="M34" s="177"/>
     </row>
     <row r="35" spans="1:14" ht="13.5" customHeight="1">
-      <c r="A35" s="214" t="s">
+      <c r="A35" s="176" t="s">
         <v>113</v>
       </c>
-      <c r="B35" s="215"/>
-      <c r="C35" s="215"/>
-      <c r="D35" s="215"/>
-      <c r="E35" s="215"/>
-      <c r="F35" s="215"/>
-      <c r="G35" s="215"/>
-      <c r="H35" s="215"/>
-      <c r="I35" s="215"/>
-      <c r="J35" s="215"/>
-      <c r="K35" s="215"/>
-      <c r="L35" s="215"/>
-      <c r="M35" s="215"/>
+      <c r="B35" s="177"/>
+      <c r="C35" s="177"/>
+      <c r="D35" s="177"/>
+      <c r="E35" s="177"/>
+      <c r="F35" s="177"/>
+      <c r="G35" s="177"/>
+      <c r="H35" s="177"/>
+      <c r="I35" s="177"/>
+      <c r="J35" s="177"/>
+      <c r="K35" s="177"/>
+      <c r="L35" s="177"/>
+      <c r="M35" s="177"/>
     </row>
     <row r="36" spans="1:14" ht="15.75" customHeight="1">
       <c r="A36" s="21"/>
@@ -3797,15 +3801,15 @@
       <c r="C36" s="106" t="s">
         <v>77</v>
       </c>
-      <c r="D36" s="209"/>
-      <c r="E36" s="141"/>
-      <c r="F36" s="141"/>
-      <c r="G36" s="141"/>
-      <c r="H36" s="141"/>
-      <c r="I36" s="141"/>
+      <c r="D36" s="200"/>
+      <c r="E36" s="159"/>
+      <c r="F36" s="159"/>
+      <c r="G36" s="159"/>
+      <c r="H36" s="159"/>
+      <c r="I36" s="159"/>
       <c r="K36" s="62"/>
-      <c r="L36" s="272"/>
-      <c r="M36" s="273"/>
+      <c r="L36" s="195"/>
+      <c r="M36" s="196"/>
     </row>
     <row r="37" spans="1:14">
       <c r="A37" s="21"/>
@@ -3814,33 +3818,33 @@
         <v>78</v>
       </c>
       <c r="D37" s="21"/>
-      <c r="E37" s="233"/>
-      <c r="F37" s="138"/>
-      <c r="G37" s="138"/>
-      <c r="H37" s="138"/>
-      <c r="I37" s="138"/>
+      <c r="E37" s="144"/>
+      <c r="F37" s="140"/>
+      <c r="G37" s="140"/>
+      <c r="H37" s="140"/>
+      <c r="I37" s="140"/>
       <c r="K37" s="59"/>
-      <c r="L37" s="274"/>
-      <c r="M37" s="275"/>
+      <c r="L37" s="198"/>
+      <c r="M37" s="199"/>
     </row>
     <row r="38" spans="1:14">
       <c r="A38" s="21"/>
       <c r="B38" s="21"/>
-      <c r="C38" s="245" t="s">
+      <c r="C38" s="178" t="s">
         <v>79</v>
       </c>
-      <c r="D38" s="145"/>
-      <c r="E38" s="145"/>
+      <c r="D38" s="179"/>
+      <c r="E38" s="179"/>
       <c r="F38" s="21"/>
-      <c r="G38" s="233"/>
-      <c r="H38" s="233"/>
-      <c r="I38" s="138"/>
+      <c r="G38" s="144"/>
+      <c r="H38" s="144"/>
+      <c r="I38" s="140"/>
       <c r="K38" s="62"/>
-      <c r="L38" s="274" t="str">
+      <c r="L38" s="198" t="str">
         <f>IF(SUM(L36:M37)=0, "", MROUND(SUM(L36:M37), 10))</f>
         <v/>
       </c>
-      <c r="M38" s="275"/>
+      <c r="M38" s="199"/>
     </row>
     <row r="39" spans="1:14" ht="27" customHeight="1">
       <c r="A39" s="21"/>
@@ -3853,8 +3857,8 @@
       <c r="H39" s="21"/>
       <c r="I39" s="21"/>
       <c r="J39" s="21"/>
-      <c r="K39" s="147"/>
-      <c r="L39" s="147"/>
+      <c r="K39" s="166"/>
+      <c r="L39" s="166"/>
       <c r="M39" s="21"/>
     </row>
     <row r="40" spans="1:14" ht="15" customHeight="1">
@@ -3868,10 +3872,10 @@
       <c r="H40" s="21"/>
       <c r="I40" s="21"/>
       <c r="J40" s="21"/>
-      <c r="K40" s="258" t="s">
+      <c r="K40" s="161" t="s">
         <v>80</v>
       </c>
-      <c r="L40" s="178"/>
+      <c r="L40" s="138"/>
       <c r="M40" s="21"/>
     </row>
     <row r="41" spans="1:14" ht="15.75" customHeight="1">
@@ -3885,19 +3889,19 @@
         <v>81</v>
       </c>
       <c r="H41" s="22"/>
-      <c r="I41" s="204"/>
-      <c r="J41" s="204"/>
-      <c r="K41" s="141"/>
-      <c r="L41" s="141"/>
+      <c r="I41" s="158"/>
+      <c r="J41" s="158"/>
+      <c r="K41" s="159"/>
+      <c r="L41" s="159"/>
       <c r="M41" s="21"/>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
-      <c r="A42" s="248" t="s">
+      <c r="A42" s="182" t="s">
         <v>104</v>
       </c>
-      <c r="B42" s="248"/>
-      <c r="C42" s="248"/>
-      <c r="D42" s="248"/>
+      <c r="B42" s="182"/>
+      <c r="C42" s="182"/>
+      <c r="D42" s="182"/>
       <c r="E42" s="114"/>
       <c r="F42" s="106" t="s">
         <v>101</v>
@@ -3906,13 +3910,13 @@
       <c r="H42" s="117">
         <v>20</v>
       </c>
-      <c r="I42" s="222"/>
-      <c r="J42" s="222"/>
-      <c r="K42" s="235" t="s">
+      <c r="I42" s="203"/>
+      <c r="J42" s="203"/>
+      <c r="K42" s="197" t="s">
         <v>114</v>
       </c>
-      <c r="L42" s="235"/>
-      <c r="M42" s="235"/>
+      <c r="L42" s="197"/>
+      <c r="M42" s="197"/>
       <c r="N42" s="21"/>
     </row>
     <row r="43" spans="1:14" ht="15.6" customHeight="1">
@@ -3929,23 +3933,23 @@
         <v>102</v>
       </c>
       <c r="I43" s="128"/>
-      <c r="J43" s="223"/>
-      <c r="K43" s="223"/>
-      <c r="L43" s="223"/>
-      <c r="M43" s="223"/>
+      <c r="J43" s="204"/>
+      <c r="K43" s="204"/>
+      <c r="L43" s="204"/>
+      <c r="M43" s="204"/>
     </row>
     <row r="44" spans="1:14">
-      <c r="A44" s="130">
+      <c r="A44" s="129">
         <v>20</v>
       </c>
       <c r="B44" s="121"/>
-      <c r="C44" s="130" t="s">
+      <c r="C44" s="129" t="s">
         <v>103</v>
       </c>
-      <c r="D44" s="213"/>
-      <c r="E44" s="213"/>
-      <c r="F44" s="213"/>
-      <c r="G44" s="213"/>
+      <c r="D44" s="201"/>
+      <c r="E44" s="201"/>
+      <c r="F44" s="201"/>
+      <c r="G44" s="201"/>
       <c r="H44" s="127" t="s">
         <v>111</v>
       </c>
@@ -3965,11 +3969,11 @@
       <c r="G45" s="21"/>
       <c r="H45" s="21"/>
       <c r="I45" s="21"/>
-      <c r="J45" s="277" t="s">
+      <c r="J45" s="167" t="s">
         <v>121</v>
       </c>
-      <c r="K45" s="277"/>
-      <c r="L45" s="277"/>
+      <c r="K45" s="167"/>
+      <c r="L45" s="167"/>
       <c r="M45" s="21"/>
     </row>
     <row r="46" spans="1:14">
@@ -3981,50 +3985,50 @@
       <c r="F46" s="21"/>
       <c r="G46" s="21"/>
       <c r="H46" s="21"/>
-      <c r="I46" s="276" t="s">
+      <c r="I46" s="202" t="s">
         <v>120</v>
       </c>
-      <c r="J46" s="276"/>
-      <c r="K46" s="276"/>
-      <c r="L46" s="276"/>
-      <c r="M46" s="276"/>
+      <c r="J46" s="202"/>
+      <c r="K46" s="202"/>
+      <c r="L46" s="202"/>
+      <c r="M46" s="202"/>
     </row>
     <row r="47" spans="1:14" ht="15" customHeight="1">
-      <c r="A47" s="228" t="s">
+      <c r="A47" s="184" t="s">
         <v>82</v>
       </c>
-      <c r="B47" s="145"/>
-      <c r="C47" s="145"/>
-      <c r="D47" s="145"/>
-      <c r="E47" s="145"/>
+      <c r="B47" s="179"/>
+      <c r="C47" s="179"/>
+      <c r="D47" s="179"/>
+      <c r="E47" s="179"/>
       <c r="F47" s="21"/>
       <c r="G47" s="21"/>
       <c r="H47" s="21"/>
       <c r="I47" s="25"/>
-      <c r="J47" s="277" t="s">
+      <c r="J47" s="167" t="s">
         <v>122</v>
       </c>
-      <c r="K47" s="277"/>
-      <c r="L47" s="277"/>
+      <c r="K47" s="167"/>
+      <c r="L47" s="167"/>
       <c r="M47" s="21"/>
     </row>
     <row r="48" spans="1:14" ht="15" customHeight="1">
-      <c r="A48" s="228" t="s">
+      <c r="A48" s="184" t="s">
         <v>83</v>
       </c>
-      <c r="B48" s="145"/>
-      <c r="C48" s="145"/>
-      <c r="D48" s="145"/>
-      <c r="E48" s="145"/>
+      <c r="B48" s="179"/>
+      <c r="C48" s="179"/>
+      <c r="D48" s="179"/>
+      <c r="E48" s="179"/>
       <c r="F48" s="21"/>
       <c r="G48" s="21"/>
       <c r="H48" s="21"/>
       <c r="I48" s="21"/>
-      <c r="J48" s="278" t="s">
+      <c r="J48" s="186" t="s">
         <v>84</v>
       </c>
-      <c r="K48" s="278"/>
-      <c r="L48" s="278"/>
+      <c r="K48" s="186"/>
+      <c r="L48" s="186"/>
       <c r="M48" s="21"/>
     </row>
     <row r="49" spans="1:27">
@@ -4038,62 +4042,62 @@
       <c r="H49" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="I49" s="204"/>
-      <c r="J49" s="204"/>
-      <c r="K49" s="141"/>
-      <c r="L49" s="141"/>
+      <c r="I49" s="158"/>
+      <c r="J49" s="158"/>
+      <c r="K49" s="159"/>
+      <c r="L49" s="159"/>
       <c r="M49" s="21"/>
     </row>
     <row r="50" spans="1:27">
-      <c r="A50" s="166"/>
-      <c r="B50" s="145"/>
-      <c r="C50" s="145"/>
-      <c r="D50" s="145"/>
-      <c r="E50" s="145"/>
-      <c r="F50" s="145"/>
-      <c r="G50" s="145"/>
-      <c r="H50" s="145"/>
-      <c r="I50" s="145"/>
-      <c r="J50" s="145"/>
-      <c r="K50" s="145"/>
-      <c r="L50" s="145"/>
-      <c r="M50" s="145"/>
+      <c r="A50" s="194"/>
+      <c r="B50" s="179"/>
+      <c r="C50" s="179"/>
+      <c r="D50" s="179"/>
+      <c r="E50" s="179"/>
+      <c r="F50" s="179"/>
+      <c r="G50" s="179"/>
+      <c r="H50" s="179"/>
+      <c r="I50" s="179"/>
+      <c r="J50" s="179"/>
+      <c r="K50" s="179"/>
+      <c r="L50" s="179"/>
+      <c r="M50" s="179"/>
     </row>
     <row r="51" spans="1:27" ht="21" customHeight="1">
-      <c r="A51" s="250"/>
-      <c r="B51" s="178"/>
-      <c r="C51" s="178"/>
-      <c r="D51" s="178"/>
-      <c r="E51" s="178"/>
-      <c r="F51" s="178"/>
-      <c r="G51" s="178"/>
-      <c r="H51" s="178"/>
-      <c r="I51" s="178"/>
-      <c r="J51" s="178"/>
-      <c r="K51" s="178"/>
-      <c r="L51" s="178"/>
-      <c r="M51" s="178"/>
+      <c r="A51" s="137"/>
+      <c r="B51" s="138"/>
+      <c r="C51" s="138"/>
+      <c r="D51" s="138"/>
+      <c r="E51" s="138"/>
+      <c r="F51" s="138"/>
+      <c r="G51" s="138"/>
+      <c r="H51" s="138"/>
+      <c r="I51" s="138"/>
+      <c r="J51" s="138"/>
+      <c r="K51" s="138"/>
+      <c r="L51" s="138"/>
+      <c r="M51" s="138"/>
     </row>
     <row r="52" spans="1:27">
-      <c r="A52" s="208"/>
-      <c r="B52" s="145"/>
-      <c r="C52" s="145"/>
-      <c r="D52" s="145"/>
-      <c r="E52" s="145"/>
-      <c r="F52" s="145"/>
-      <c r="G52" s="145"/>
-      <c r="H52" s="145"/>
-      <c r="I52" s="145"/>
-      <c r="J52" s="145"/>
-      <c r="K52" s="145"/>
-      <c r="L52" s="145"/>
-      <c r="M52" s="145"/>
+      <c r="A52" s="214"/>
+      <c r="B52" s="179"/>
+      <c r="C52" s="179"/>
+      <c r="D52" s="179"/>
+      <c r="E52" s="179"/>
+      <c r="F52" s="179"/>
+      <c r="G52" s="179"/>
+      <c r="H52" s="179"/>
+      <c r="I52" s="179"/>
+      <c r="J52" s="179"/>
+      <c r="K52" s="179"/>
+      <c r="L52" s="179"/>
+      <c r="M52" s="179"/>
     </row>
     <row r="53" spans="1:27">
-      <c r="A53" s="244" t="s">
+      <c r="A53" s="174" t="s">
         <v>85</v>
       </c>
-      <c r="B53" s="141"/>
+      <c r="B53" s="159"/>
       <c r="C53" s="24"/>
       <c r="D53" s="24" t="s">
         <v>86</v>
@@ -4105,21 +4109,21 @@
       </c>
       <c r="H53" s="24"/>
       <c r="I53" s="24"/>
-      <c r="J53" s="204" t="s">
+      <c r="J53" s="158" t="s">
         <v>87</v>
       </c>
-      <c r="K53" s="204"/>
+      <c r="K53" s="158"/>
       <c r="L53" s="21"/>
       <c r="M53" s="61" t="s">
         <v>88</v>
       </c>
-      <c r="O53" s="160"/>
-      <c r="P53" s="145"/>
+      <c r="O53" s="206"/>
+      <c r="P53" s="179"/>
       <c r="Q53" s="21"/>
       <c r="R53" s="21"/>
       <c r="S53" s="21"/>
-      <c r="T53" s="160"/>
-      <c r="U53" s="145"/>
+      <c r="T53" s="206"/>
+      <c r="U53" s="179"/>
       <c r="V53" s="21"/>
       <c r="W53" s="21"/>
       <c r="X53" s="21"/>
@@ -4128,8 +4132,8 @@
       <c r="AA53" s="60"/>
     </row>
     <row r="54" spans="1:27">
-      <c r="A54" s="147"/>
-      <c r="B54" s="141"/>
+      <c r="A54" s="166"/>
+      <c r="B54" s="159"/>
       <c r="C54" s="97"/>
       <c r="D54" s="99"/>
       <c r="E54" s="97"/>
@@ -4137,16 +4141,16 @@
       <c r="G54" s="102"/>
       <c r="H54" s="116"/>
       <c r="I54" s="98"/>
-      <c r="J54" s="131"/>
-      <c r="K54" s="132"/>
+      <c r="J54" s="130"/>
+      <c r="K54" s="131"/>
       <c r="L54" s="96" t="s">
         <v>105</v>
       </c>
       <c r="M54" s="102"/>
     </row>
     <row r="55" spans="1:27">
-      <c r="A55" s="212"/>
-      <c r="B55" s="138"/>
+      <c r="A55" s="188"/>
+      <c r="B55" s="140"/>
       <c r="C55" s="97"/>
       <c r="D55" s="100"/>
       <c r="E55" s="97"/>
@@ -4154,16 +4158,16 @@
       <c r="G55" s="102"/>
       <c r="H55" s="116"/>
       <c r="I55" s="98"/>
-      <c r="J55" s="131"/>
-      <c r="K55" s="132"/>
+      <c r="J55" s="130"/>
+      <c r="K55" s="131"/>
       <c r="L55" s="96" t="s">
         <v>105</v>
       </c>
       <c r="M55" s="102"/>
     </row>
     <row r="56" spans="1:27">
-      <c r="A56" s="212"/>
-      <c r="B56" s="138"/>
+      <c r="A56" s="188"/>
+      <c r="B56" s="140"/>
       <c r="C56" s="97"/>
       <c r="D56" s="101"/>
       <c r="E56" s="97"/>
@@ -4171,16 +4175,16 @@
       <c r="G56" s="102"/>
       <c r="H56" s="116"/>
       <c r="I56" s="98"/>
-      <c r="J56" s="131"/>
-      <c r="K56" s="132"/>
+      <c r="J56" s="130"/>
+      <c r="K56" s="131"/>
       <c r="L56" s="96" t="s">
         <v>105</v>
       </c>
       <c r="M56" s="102"/>
     </row>
     <row r="57" spans="1:27">
-      <c r="A57" s="212"/>
-      <c r="B57" s="138"/>
+      <c r="A57" s="188"/>
+      <c r="B57" s="140"/>
       <c r="C57" s="97"/>
       <c r="D57" s="101"/>
       <c r="E57" s="97"/>
@@ -4188,8 +4192,8 @@
       <c r="G57" s="102"/>
       <c r="H57" s="116"/>
       <c r="I57" s="98"/>
-      <c r="J57" s="131"/>
-      <c r="K57" s="132"/>
+      <c r="J57" s="130"/>
+      <c r="K57" s="131"/>
       <c r="L57" s="96" t="s">
         <v>105</v>
       </c>
@@ -4204,9 +4208,9 @@
         <v/>
       </c>
       <c r="H58" s="116"/>
-      <c r="I58" s="166"/>
-      <c r="J58" s="166"/>
-      <c r="K58" s="145"/>
+      <c r="I58" s="194"/>
+      <c r="J58" s="194"/>
+      <c r="K58" s="179"/>
       <c r="L58" s="108" t="s">
         <v>31</v>
       </c>
@@ -4216,41 +4220,41 @@
       </c>
     </row>
     <row r="59" spans="1:27">
-      <c r="A59" s="230" t="s">
+      <c r="A59" s="191" t="s">
         <v>89</v>
       </c>
-      <c r="B59" s="231"/>
-      <c r="C59" s="231"/>
-      <c r="D59" s="237"/>
-      <c r="E59" s="138"/>
-      <c r="F59" s="138"/>
-      <c r="G59" s="138"/>
-      <c r="H59" s="138"/>
-      <c r="I59" s="138"/>
-      <c r="J59" s="138"/>
-      <c r="K59" s="138"/>
-      <c r="L59" s="138"/>
-      <c r="M59" s="138"/>
+      <c r="B59" s="192"/>
+      <c r="C59" s="192"/>
+      <c r="D59" s="216"/>
+      <c r="E59" s="140"/>
+      <c r="F59" s="140"/>
+      <c r="G59" s="140"/>
+      <c r="H59" s="140"/>
+      <c r="I59" s="140"/>
+      <c r="J59" s="140"/>
+      <c r="K59" s="140"/>
+      <c r="L59" s="140"/>
+      <c r="M59" s="140"/>
     </row>
     <row r="60" spans="1:27" ht="21.75" customHeight="1">
-      <c r="A60" s="238" t="s">
+      <c r="A60" s="217" t="s">
         <v>90</v>
       </c>
-      <c r="B60" s="175"/>
-      <c r="C60" s="175"/>
+      <c r="B60" s="218"/>
+      <c r="C60" s="218"/>
       <c r="G60" s="122" t="s">
         <v>91</v>
       </c>
-      <c r="I60" s="176"/>
-      <c r="J60" s="176"/>
-      <c r="K60" s="145"/>
+      <c r="I60" s="185"/>
+      <c r="J60" s="185"/>
+      <c r="K60" s="179"/>
     </row>
     <row r="61" spans="1:27" ht="23.25" customHeight="1">
-      <c r="A61" s="202" t="s">
+      <c r="A61" s="209" t="s">
         <v>123</v>
       </c>
-      <c r="B61" s="203"/>
-      <c r="C61" s="203"/>
+      <c r="B61" s="210"/>
+      <c r="C61" s="210"/>
       <c r="D61" s="21"/>
       <c r="E61" s="21"/>
       <c r="F61" s="21"/>
@@ -4258,16 +4262,16 @@
       <c r="H61" s="21"/>
       <c r="I61" s="21"/>
       <c r="J61" s="21"/>
-      <c r="K61" s="208"/>
-      <c r="L61" s="145"/>
+      <c r="K61" s="214"/>
+      <c r="L61" s="179"/>
       <c r="M61" s="21"/>
     </row>
     <row r="62" spans="1:27" ht="21" customHeight="1">
-      <c r="A62" s="278" t="s">
+      <c r="A62" s="186" t="s">
         <v>92</v>
       </c>
-      <c r="B62" s="279"/>
-      <c r="C62" s="279"/>
+      <c r="B62" s="187"/>
+      <c r="C62" s="187"/>
       <c r="D62" s="21"/>
       <c r="E62" s="21"/>
       <c r="F62" s="21"/>
@@ -4275,10 +4279,10 @@
       <c r="H62" s="21"/>
       <c r="I62" s="21"/>
       <c r="J62" s="21"/>
-      <c r="K62" s="226" t="s">
+      <c r="K62" s="189" t="s">
         <v>92</v>
       </c>
-      <c r="L62" s="227"/>
+      <c r="L62" s="190"/>
       <c r="M62" s="21"/>
     </row>
     <row r="63" spans="1:27">
@@ -4294,8 +4298,8 @@
       <c r="J63" s="109" t="s">
         <v>93</v>
       </c>
-      <c r="K63" s="207"/>
-      <c r="L63" s="178"/>
+      <c r="K63" s="213"/>
+      <c r="L63" s="138"/>
       <c r="M63" s="21"/>
     </row>
     <row r="64" spans="1:27">
@@ -4309,10 +4313,10 @@
       <c r="H64" s="21"/>
       <c r="I64" s="21"/>
       <c r="J64" s="21"/>
-      <c r="K64" s="200" t="s">
+      <c r="K64" s="207" t="s">
         <v>94</v>
       </c>
-      <c r="L64" s="201"/>
+      <c r="L64" s="208"/>
       <c r="M64" s="21"/>
     </row>
     <row r="65" spans="1:13">
@@ -4324,12 +4328,12 @@
       <c r="F65" s="57"/>
       <c r="G65" s="57"/>
       <c r="H65" s="57"/>
-      <c r="I65" s="133"/>
-      <c r="J65" s="133" t="s">
+      <c r="I65" s="132"/>
+      <c r="J65" s="132" t="s">
         <v>95</v>
       </c>
-      <c r="K65" s="204"/>
-      <c r="L65" s="141"/>
+      <c r="K65" s="158"/>
+      <c r="L65" s="159"/>
       <c r="M65" s="57"/>
     </row>
     <row r="66" spans="1:13" ht="3" customHeight="1">
@@ -4348,19 +4352,19 @@
       <c r="M66" s="58"/>
     </row>
     <row r="67" spans="1:13">
-      <c r="A67" s="240" t="s">
+      <c r="A67" s="219" t="s">
         <v>96</v>
       </c>
-      <c r="B67" s="240"/>
-      <c r="C67" s="240"/>
-      <c r="D67" s="240"/>
-      <c r="E67" s="147"/>
-      <c r="F67" s="147"/>
-      <c r="G67" s="147"/>
-      <c r="H67" s="147"/>
-      <c r="I67" s="147"/>
-      <c r="J67" s="147"/>
-      <c r="K67" s="147"/>
+      <c r="B67" s="219"/>
+      <c r="C67" s="219"/>
+      <c r="D67" s="219"/>
+      <c r="E67" s="166"/>
+      <c r="F67" s="166"/>
+      <c r="G67" s="166"/>
+      <c r="H67" s="166"/>
+      <c r="I67" s="166"/>
+      <c r="J67" s="166"/>
+      <c r="K67" s="166"/>
       <c r="L67" s="124"/>
       <c r="M67" s="69" t="s">
         <v>97</v>
@@ -4378,12 +4382,12 @@
       <c r="G68" s="57"/>
       <c r="H68" s="58"/>
       <c r="I68" s="71"/>
-      <c r="J68" s="241" t="s">
+      <c r="J68" s="220" t="s">
         <v>98</v>
       </c>
-      <c r="K68" s="241"/>
-      <c r="L68" s="241"/>
-      <c r="M68" s="241"/>
+      <c r="K68" s="220"/>
+      <c r="L68" s="220"/>
+      <c r="M68" s="220"/>
     </row>
     <row r="69" spans="1:13">
       <c r="A69" s="125" t="s">
@@ -4394,78 +4398,158 @@
         <v>107</v>
       </c>
       <c r="D69" s="126"/>
-      <c r="E69" s="150"/>
-      <c r="F69" s="141"/>
-      <c r="G69" s="141"/>
-      <c r="H69" s="141"/>
-      <c r="I69" s="141"/>
-      <c r="J69" s="242" t="s">
+      <c r="E69" s="212"/>
+      <c r="F69" s="159"/>
+      <c r="G69" s="159"/>
+      <c r="H69" s="159"/>
+      <c r="I69" s="159"/>
+      <c r="J69" s="221" t="s">
         <v>108</v>
       </c>
-      <c r="K69" s="242"/>
-      <c r="L69" s="242"/>
-      <c r="M69" s="242"/>
+      <c r="K69" s="221"/>
+      <c r="L69" s="221"/>
+      <c r="M69" s="221"/>
     </row>
     <row r="70" spans="1:13">
-      <c r="A70" s="69" t="s">
+      <c r="A70" s="125" t="s">
+        <v>124</v>
+      </c>
+      <c r="B70" s="279"/>
+      <c r="C70" s="280" t="s">
+        <v>125</v>
+      </c>
+      <c r="D70" s="124"/>
+      <c r="E70" s="281" t="s">
+        <v>126</v>
+      </c>
+      <c r="F70" s="281"/>
+      <c r="G70" s="212"/>
+      <c r="H70" s="212"/>
+      <c r="I70" s="212"/>
+      <c r="J70" s="212"/>
+      <c r="K70" s="212"/>
+      <c r="L70" s="212"/>
+      <c r="M70" s="212"/>
+    </row>
+    <row r="71" spans="1:13">
+      <c r="A71" s="69" t="s">
         <v>109</v>
       </c>
-      <c r="B70" s="69"/>
-      <c r="C70" s="69"/>
-      <c r="D70" s="69"/>
-      <c r="E70" s="102"/>
-      <c r="G70" s="69" t="s">
+      <c r="B71" s="69"/>
+      <c r="C71" s="69"/>
+      <c r="D71" s="69"/>
+      <c r="E71" s="136"/>
+      <c r="G71" s="69" t="s">
         <v>110</v>
       </c>
-      <c r="H70" s="243"/>
-      <c r="I70" s="243"/>
-      <c r="J70" s="118"/>
-      <c r="K70" s="70" t="s">
+      <c r="H71" s="222"/>
+      <c r="I71" s="222"/>
+      <c r="J71" s="118"/>
+      <c r="K71" s="70" t="s">
         <v>100</v>
       </c>
-      <c r="L70" s="205" t="str">
-        <f>IF(SUM(I70,E70)=0, "", MROUND(SUM(I70,E70), 10))</f>
+      <c r="L71" s="211" t="str">
+        <f>IF(SUM(H71,E71)=0, "", MROUND(SUM(H71,E71), 10))</f>
         <v/>
       </c>
-      <c r="M70" s="141"/>
-    </row>
-    <row r="71" spans="1:13">
-      <c r="A71" s="202"/>
-      <c r="B71" s="203"/>
-      <c r="C71" s="203"/>
-      <c r="D71" s="203"/>
-      <c r="E71" s="129"/>
-      <c r="H71" s="239"/>
-      <c r="I71" s="239"/>
-      <c r="L71" s="236"/>
-      <c r="M71" s="178"/>
+      <c r="M71" s="159"/>
+    </row>
+    <row r="72" spans="1:13">
+      <c r="A72" s="209"/>
+      <c r="B72" s="210"/>
+      <c r="C72" s="210"/>
+      <c r="D72" s="210"/>
+      <c r="E72" s="113"/>
+      <c r="H72" s="215"/>
+      <c r="I72" s="215"/>
+      <c r="L72" s="215"/>
+      <c r="M72" s="138"/>
     </row>
   </sheetData>
-  <mergeCells count="129">
+  <mergeCells count="131">
+    <mergeCell ref="F3:L3"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="F10:L10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="A72:D72"/>
+    <mergeCell ref="O53:P53"/>
+    <mergeCell ref="K65:L65"/>
+    <mergeCell ref="L71:M71"/>
+    <mergeCell ref="E69:I69"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="K63:L63"/>
+    <mergeCell ref="A52:M52"/>
+    <mergeCell ref="I58:K58"/>
+    <mergeCell ref="L72:M72"/>
+    <mergeCell ref="D59:M59"/>
+    <mergeCell ref="K61:L61"/>
+    <mergeCell ref="A60:C60"/>
+    <mergeCell ref="E67:K67"/>
+    <mergeCell ref="A61:C61"/>
+    <mergeCell ref="H72:I72"/>
+    <mergeCell ref="A67:D67"/>
+    <mergeCell ref="J68:M68"/>
+    <mergeCell ref="J69:M69"/>
+    <mergeCell ref="H71:I71"/>
+    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="G70:M70"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A31:L31"/>
     <mergeCell ref="J48:L48"/>
-    <mergeCell ref="A51:M51"/>
-    <mergeCell ref="A29:D29"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="A13:D13"/>
-    <mergeCell ref="E37:I37"/>
-    <mergeCell ref="A18:M18"/>
-    <mergeCell ref="H19:J20"/>
-    <mergeCell ref="H26:J27"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="H21:J21"/>
-    <mergeCell ref="H22:J22"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="H13:J13"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="I41:L41"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="K40:L40"/>
-    <mergeCell ref="M10:M11"/>
-    <mergeCell ref="A12:D12"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="K39:L39"/>
-    <mergeCell ref="J45:L45"/>
-    <mergeCell ref="J47:L47"/>
+    <mergeCell ref="T53:U53"/>
+    <mergeCell ref="K64:L64"/>
+    <mergeCell ref="I49:L49"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="D36:I36"/>
+    <mergeCell ref="A25:M25"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="A54:B54"/>
+    <mergeCell ref="A56:B56"/>
+    <mergeCell ref="D44:G44"/>
+    <mergeCell ref="A34:M34"/>
+    <mergeCell ref="E26:G27"/>
+    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="I46:M46"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="J43:M43"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="I60:K60"/>
+    <mergeCell ref="A3:D4"/>
+    <mergeCell ref="A62:C62"/>
+    <mergeCell ref="A55:B55"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="A57:B57"/>
+    <mergeCell ref="K62:L62"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="A50:M50"/>
+    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="G38:I38"/>
+    <mergeCell ref="A30:D30"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A24:L24"/>
+    <mergeCell ref="L36:M36"/>
+    <mergeCell ref="K42:M42"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="A7:D7"/>
     <mergeCell ref="A10:D11"/>
@@ -4490,87 +4574,30 @@
     <mergeCell ref="A42:D42"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="I60:K60"/>
-    <mergeCell ref="A3:D4"/>
-    <mergeCell ref="A62:C62"/>
-    <mergeCell ref="A55:B55"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="A57:B57"/>
-    <mergeCell ref="K62:L62"/>
-    <mergeCell ref="A47:E47"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A8:L8"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="A50:M50"/>
-    <mergeCell ref="A9:M9"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="G38:I38"/>
-    <mergeCell ref="A30:D30"/>
-    <mergeCell ref="A15:L15"/>
-    <mergeCell ref="A24:L24"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="K42:M42"/>
+    <mergeCell ref="A51:M51"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="E37:I37"/>
+    <mergeCell ref="A18:M18"/>
+    <mergeCell ref="H19:J20"/>
+    <mergeCell ref="H26:J27"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="H21:J21"/>
+    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="I41:L41"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="K40:L40"/>
+    <mergeCell ref="M10:M11"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="K39:L39"/>
+    <mergeCell ref="J45:L45"/>
+    <mergeCell ref="J47:L47"/>
     <mergeCell ref="A14:D14"/>
-    <mergeCell ref="I49:L49"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="D36:I36"/>
-    <mergeCell ref="A25:M25"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="A54:B54"/>
-    <mergeCell ref="A56:B56"/>
-    <mergeCell ref="D44:G44"/>
-    <mergeCell ref="A34:M34"/>
-    <mergeCell ref="E26:G27"/>
-    <mergeCell ref="L38:M38"/>
-    <mergeCell ref="I46:M46"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="J43:M43"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="A28:D28"/>
-    <mergeCell ref="A31:L31"/>
-    <mergeCell ref="T53:U53"/>
-    <mergeCell ref="K64:L64"/>
-    <mergeCell ref="A71:D71"/>
-    <mergeCell ref="O53:P53"/>
-    <mergeCell ref="K65:L65"/>
-    <mergeCell ref="L70:M70"/>
-    <mergeCell ref="E69:I69"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="K63:L63"/>
-    <mergeCell ref="A52:M52"/>
-    <mergeCell ref="I58:K58"/>
-    <mergeCell ref="L71:M71"/>
-    <mergeCell ref="D59:M59"/>
-    <mergeCell ref="K61:L61"/>
-    <mergeCell ref="A60:C60"/>
-    <mergeCell ref="E67:K67"/>
-    <mergeCell ref="A61:C61"/>
-    <mergeCell ref="H71:I71"/>
-    <mergeCell ref="A67:D67"/>
-    <mergeCell ref="J68:M68"/>
-    <mergeCell ref="J69:M69"/>
-    <mergeCell ref="H70:I70"/>
-    <mergeCell ref="M26:M27"/>
-    <mergeCell ref="F3:L3"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="F6:G6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="F10:L10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="H5:J5"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>

</xml_diff>